<commit_message>
code change for time series, new data for Jan and Feb 2026
</commit_message>
<xml_diff>
--- a/exh1.xlsx
+++ b/exh1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\econ019fs\ftd53\TDSB2\Internet\Current\Press-Release\current_press_release\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2DA8483E-753D-4671-899C-1FAEDD181EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{59223F66-91E5-4506-AB12-68DB50A839D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8510" yWindow="-10910" windowWidth="19420" windowHeight="10300" xr2:uid="{ECAC4F86-B477-44C2-B924-F390EE5D3FF6}"/>
+    <workbookView xWindow="9876" yWindow="-13068" windowWidth="23256" windowHeight="12456" xr2:uid="{662D1F84-5564-422C-825A-E32495AEA09F}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <externalReference r:id="rId2"/>
     <externalReference r:id="rId3"/>
     <externalReference r:id="rId4"/>
+    <externalReference r:id="rId5"/>
   </externalReferences>
   <definedNames>
     <definedName name="exhibit1">#REF!</definedName>
@@ -45,7 +46,8 @@
     <definedName name="gsfimpcountries">'[2]SF Goods Imports'!$A$4:$S$4</definedName>
     <definedName name="gsfimpquarters">'[2]SF Goods Imports'!$A$4:$A$500</definedName>
     <definedName name="PRINT">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'1'!$A$1:$J$53</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'1'!$A$1:$J$55</definedName>
+    <definedName name="_xlnm.Print_Area">#REF!</definedName>
     <definedName name="qlookup">[2]Codes!$A$22:$B$25</definedName>
     <definedName name="snsaexp">'[2]NSA Services Exports'!$A$4:$S$500</definedName>
     <definedName name="snsaexpcountries">'[2]NSA Services Exports'!$A$4:$S$4</definedName>
@@ -53,21 +55,21 @@
     <definedName name="snsaimp">'[2]NSA Services Imports'!$A$4:$S$500</definedName>
     <definedName name="snsaimpcountries">'[2]NSA Services Imports'!$A$4:$S$4</definedName>
     <definedName name="snsaimpquarters">'[2]NSA Services Imports'!$A$4:$A$500</definedName>
-    <definedName name="ssa">'[3]SA Services Imports Forced'!$A$4:$S$4</definedName>
+    <definedName name="ssa">'[4]SA Services Imports Forced'!$A$4:$S$4</definedName>
     <definedName name="ssaexp">'[2]SA Services Exports Forced'!$A$4:$S$500</definedName>
     <definedName name="ssaexpcountries">'[2]SA Services Exports Forced'!$A$4:$S$4</definedName>
     <definedName name="ssaexpquarters">'[2]SA Services Exports Forced'!$A$4:$A$500</definedName>
     <definedName name="ssaimp">'[2]SA Services Imports Forced'!$A$4:$S$500</definedName>
     <definedName name="ssaimpcountries">'[2]SA Services Imports Forced'!$A$4:$S$4</definedName>
     <definedName name="ssaimpquarters">'[2]SA Services Imports Forced'!$A$4:$A$500</definedName>
-    <definedName name="ssas">'[3]SA Services Imports Forced'!$A$4:$A$500</definedName>
-    <definedName name="ssf">'[3]SF Services Exports'!$A$4:$S$4</definedName>
-    <definedName name="ssfe">'[3]SF Services Exports'!$A$4:$A$500</definedName>
+    <definedName name="ssas">'[4]SA Services Imports Forced'!$A$4:$A$500</definedName>
+    <definedName name="ssf">'[4]SF Services Exports'!$A$4:$S$4</definedName>
+    <definedName name="ssfe">'[4]SF Services Exports'!$A$4:$A$500</definedName>
     <definedName name="ssfexp">'[2]SF Services Exports'!$A$4:$S$500</definedName>
     <definedName name="ssfexpcountries">'[2]SF Services Exports'!$A$4:$S$4</definedName>
     <definedName name="ssfexpquarters">'[2]SF Services Exports'!$A$4:$A$500</definedName>
-    <definedName name="ssfi">'[3]SF Services Imports'!$A$4:$S$500</definedName>
-    <definedName name="ssfim">'[3]SF Services Imports'!$A$4:$A$500</definedName>
+    <definedName name="ssfi">'[4]SF Services Imports'!$A$4:$S$500</definedName>
+    <definedName name="ssfim">'[4]SF Services Imports'!$A$4:$A$500</definedName>
     <definedName name="ssfimp">'[2]SF Services Imports'!$A$4:$S$500</definedName>
     <definedName name="ssfimpcountries">'[2]SF Services Imports'!$A$4:$S$4</definedName>
     <definedName name="ssfimpquarters">'[2]SF Services Imports'!$A$4:$A$500</definedName>
@@ -94,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="47">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -105,7 +107,7 @@
     <t>Exhibit 1. U.S. International Trade in Goods and Services</t>
   </si>
   <si>
-    <t>In millions of dollars. Details may not equal totals due to seasonal adjustment and rounding.  (R) - Revised.</t>
+    <t>In millions of dollars. Details may not equal totals due to seasonal adjustment and rounding. (R) - Revised.</t>
   </si>
   <si>
     <t>Period</t>
@@ -129,10 +131,13 @@
     <t>Services</t>
   </si>
   <si>
-    <t>2023</t>
+    <t>2024</t>
   </si>
   <si>
-    <t>Jan.- Dec.</t>
+    <t>Jan. - Dec.</t>
+  </si>
+  <si>
+    <t>Jan. -</t>
   </si>
   <si>
     <t>January</t>
@@ -171,46 +176,58 @@
     <t>December</t>
   </si>
   <si>
-    <t>2024</t>
-  </si>
-  <si>
     <t>2025</t>
   </si>
   <si>
-    <t xml:space="preserve">January (R) </t>
+    <t>Jan. - Dec. (R)</t>
   </si>
   <si>
-    <t xml:space="preserve">February (R) </t>
+    <t>Jan. - (R)</t>
   </si>
   <si>
-    <t xml:space="preserve">March (R) </t>
+    <t>January (R)</t>
   </si>
   <si>
-    <t xml:space="preserve">April (R) </t>
+    <t>February (R)</t>
   </si>
   <si>
-    <t xml:space="preserve">May (R) </t>
+    <t>March (R)</t>
   </si>
   <si>
-    <t xml:space="preserve">June (R) </t>
+    <t>April (R)</t>
   </si>
   <si>
-    <t xml:space="preserve">July (R) </t>
+    <t>May (R)</t>
   </si>
   <si>
-    <t xml:space="preserve">August (R) </t>
+    <t>June (R)</t>
   </si>
   <si>
-    <t xml:space="preserve">September (R) </t>
+    <t>July (R)</t>
   </si>
   <si>
-    <t xml:space="preserve">October (R) </t>
+    <t>August (R)</t>
   </si>
   <si>
-    <t xml:space="preserve">November (R) </t>
+    <t>September (R)</t>
   </si>
   <si>
-    <t>November data as published last month:</t>
+    <t>October (R)</t>
+  </si>
+  <si>
+    <t>November (R)</t>
+  </si>
+  <si>
+    <t>December (R)</t>
+  </si>
+  <si>
+    <t>2026</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>December data as published last month:</t>
   </si>
   <si>
     <t>(1) Data are presented on a balance of payments (BOP) basis.</t>
@@ -226,7 +243,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <name val="Arial"/>
@@ -251,11 +268,6 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="16"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -292,7 +304,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -302,14 +314,14 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </left>
       <right/>
       <top style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -317,23 +329,23 @@
       <left/>
       <right/>
       <top style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -369,7 +381,9 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
+      <right style="double">
+        <color indexed="64"/>
+      </right>
       <top style="double">
         <color indexed="64"/>
       </top>
@@ -382,34 +396,6 @@
       <left style="double">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="double">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="double">
-        <color indexed="64"/>
-      </right>
-      <top style="double">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -453,7 +439,9 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
+      <right style="double">
+        <color indexed="64"/>
+      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -466,34 +454,6 @@
       <left style="double">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="double">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="double">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="double">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -550,6 +510,57 @@
       <top style="double">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="double">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -616,52 +627,10 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
+      <right/>
+      <top style="thin">
         <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="double">
-        <color indexed="64"/>
-      </right>
-      <top/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -669,7 +638,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -679,19 +648,19 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
@@ -711,10 +680,10 @@
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -722,56 +691,48 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -51447,6 +51408,70 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="1"/>
+      <sheetName val="2"/>
+      <sheetName val="3"/>
+      <sheetName val="4"/>
+      <sheetName val="5"/>
+      <sheetName val="6"/>
+      <sheetName val="7"/>
+      <sheetName val="8"/>
+      <sheetName val="9"/>
+      <sheetName val="10"/>
+      <sheetName val="11"/>
+      <sheetName val="12"/>
+      <sheetName val="13"/>
+      <sheetName val="14"/>
+      <sheetName val="14a"/>
+      <sheetName val="15"/>
+      <sheetName val="16"/>
+      <sheetName val="16a"/>
+      <sheetName val="17"/>
+      <sheetName val="17a"/>
+      <sheetName val="18"/>
+      <sheetName val="19"/>
+      <sheetName val="20"/>
+      <sheetName val="20a"/>
+      <sheetName val="20b"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+      <sheetData sheetId="21"/>
+      <sheetData sheetId="22"/>
+      <sheetData sheetId="23"/>
+      <sheetData sheetId="24"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
@@ -56915,214 +56940,214 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25ABFDD0-2079-4351-BEF6-FD45734BB2B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E2AFEB5-D527-46BB-8C88-2955EE412D12}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:HY53"/>
-  <sheetFormatPr defaultColWidth="9.69140625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:HY63"/>
+  <sheetFormatPr defaultColWidth="9.6328125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.69140625" style="2" customWidth="1"/>
-    <col min="2" max="10" width="10.69140625" style="2" customWidth="1"/>
-    <col min="11" max="256" width="9.69140625" style="3"/>
-    <col min="257" max="257" width="12.69140625" style="3" customWidth="1"/>
-    <col min="258" max="266" width="10.69140625" style="3" customWidth="1"/>
-    <col min="267" max="512" width="9.69140625" style="3"/>
-    <col min="513" max="513" width="12.69140625" style="3" customWidth="1"/>
-    <col min="514" max="522" width="10.69140625" style="3" customWidth="1"/>
-    <col min="523" max="768" width="9.69140625" style="3"/>
-    <col min="769" max="769" width="12.69140625" style="3" customWidth="1"/>
-    <col min="770" max="778" width="10.69140625" style="3" customWidth="1"/>
-    <col min="779" max="1024" width="9.69140625" style="3"/>
-    <col min="1025" max="1025" width="12.69140625" style="3" customWidth="1"/>
-    <col min="1026" max="1034" width="10.69140625" style="3" customWidth="1"/>
-    <col min="1035" max="1280" width="9.69140625" style="3"/>
-    <col min="1281" max="1281" width="12.69140625" style="3" customWidth="1"/>
-    <col min="1282" max="1290" width="10.69140625" style="3" customWidth="1"/>
-    <col min="1291" max="1536" width="9.69140625" style="3"/>
-    <col min="1537" max="1537" width="12.69140625" style="3" customWidth="1"/>
-    <col min="1538" max="1546" width="10.69140625" style="3" customWidth="1"/>
-    <col min="1547" max="1792" width="9.69140625" style="3"/>
-    <col min="1793" max="1793" width="12.69140625" style="3" customWidth="1"/>
-    <col min="1794" max="1802" width="10.69140625" style="3" customWidth="1"/>
-    <col min="1803" max="2048" width="9.69140625" style="3"/>
-    <col min="2049" max="2049" width="12.69140625" style="3" customWidth="1"/>
-    <col min="2050" max="2058" width="10.69140625" style="3" customWidth="1"/>
-    <col min="2059" max="2304" width="9.69140625" style="3"/>
-    <col min="2305" max="2305" width="12.69140625" style="3" customWidth="1"/>
-    <col min="2306" max="2314" width="10.69140625" style="3" customWidth="1"/>
-    <col min="2315" max="2560" width="9.69140625" style="3"/>
-    <col min="2561" max="2561" width="12.69140625" style="3" customWidth="1"/>
-    <col min="2562" max="2570" width="10.69140625" style="3" customWidth="1"/>
-    <col min="2571" max="2816" width="9.69140625" style="3"/>
-    <col min="2817" max="2817" width="12.69140625" style="3" customWidth="1"/>
-    <col min="2818" max="2826" width="10.69140625" style="3" customWidth="1"/>
-    <col min="2827" max="3072" width="9.69140625" style="3"/>
-    <col min="3073" max="3073" width="12.69140625" style="3" customWidth="1"/>
-    <col min="3074" max="3082" width="10.69140625" style="3" customWidth="1"/>
-    <col min="3083" max="3328" width="9.69140625" style="3"/>
-    <col min="3329" max="3329" width="12.69140625" style="3" customWidth="1"/>
-    <col min="3330" max="3338" width="10.69140625" style="3" customWidth="1"/>
-    <col min="3339" max="3584" width="9.69140625" style="3"/>
-    <col min="3585" max="3585" width="12.69140625" style="3" customWidth="1"/>
-    <col min="3586" max="3594" width="10.69140625" style="3" customWidth="1"/>
-    <col min="3595" max="3840" width="9.69140625" style="3"/>
-    <col min="3841" max="3841" width="12.69140625" style="3" customWidth="1"/>
-    <col min="3842" max="3850" width="10.69140625" style="3" customWidth="1"/>
-    <col min="3851" max="4096" width="9.69140625" style="3"/>
-    <col min="4097" max="4097" width="12.69140625" style="3" customWidth="1"/>
-    <col min="4098" max="4106" width="10.69140625" style="3" customWidth="1"/>
-    <col min="4107" max="4352" width="9.69140625" style="3"/>
-    <col min="4353" max="4353" width="12.69140625" style="3" customWidth="1"/>
-    <col min="4354" max="4362" width="10.69140625" style="3" customWidth="1"/>
-    <col min="4363" max="4608" width="9.69140625" style="3"/>
-    <col min="4609" max="4609" width="12.69140625" style="3" customWidth="1"/>
-    <col min="4610" max="4618" width="10.69140625" style="3" customWidth="1"/>
-    <col min="4619" max="4864" width="9.69140625" style="3"/>
-    <col min="4865" max="4865" width="12.69140625" style="3" customWidth="1"/>
-    <col min="4866" max="4874" width="10.69140625" style="3" customWidth="1"/>
-    <col min="4875" max="5120" width="9.69140625" style="3"/>
-    <col min="5121" max="5121" width="12.69140625" style="3" customWidth="1"/>
-    <col min="5122" max="5130" width="10.69140625" style="3" customWidth="1"/>
-    <col min="5131" max="5376" width="9.69140625" style="3"/>
-    <col min="5377" max="5377" width="12.69140625" style="3" customWidth="1"/>
-    <col min="5378" max="5386" width="10.69140625" style="3" customWidth="1"/>
-    <col min="5387" max="5632" width="9.69140625" style="3"/>
-    <col min="5633" max="5633" width="12.69140625" style="3" customWidth="1"/>
-    <col min="5634" max="5642" width="10.69140625" style="3" customWidth="1"/>
-    <col min="5643" max="5888" width="9.69140625" style="3"/>
-    <col min="5889" max="5889" width="12.69140625" style="3" customWidth="1"/>
-    <col min="5890" max="5898" width="10.69140625" style="3" customWidth="1"/>
-    <col min="5899" max="6144" width="9.69140625" style="3"/>
-    <col min="6145" max="6145" width="12.69140625" style="3" customWidth="1"/>
-    <col min="6146" max="6154" width="10.69140625" style="3" customWidth="1"/>
-    <col min="6155" max="6400" width="9.69140625" style="3"/>
-    <col min="6401" max="6401" width="12.69140625" style="3" customWidth="1"/>
-    <col min="6402" max="6410" width="10.69140625" style="3" customWidth="1"/>
-    <col min="6411" max="6656" width="9.69140625" style="3"/>
-    <col min="6657" max="6657" width="12.69140625" style="3" customWidth="1"/>
-    <col min="6658" max="6666" width="10.69140625" style="3" customWidth="1"/>
-    <col min="6667" max="6912" width="9.69140625" style="3"/>
-    <col min="6913" max="6913" width="12.69140625" style="3" customWidth="1"/>
-    <col min="6914" max="6922" width="10.69140625" style="3" customWidth="1"/>
-    <col min="6923" max="7168" width="9.69140625" style="3"/>
-    <col min="7169" max="7169" width="12.69140625" style="3" customWidth="1"/>
-    <col min="7170" max="7178" width="10.69140625" style="3" customWidth="1"/>
-    <col min="7179" max="7424" width="9.69140625" style="3"/>
-    <col min="7425" max="7425" width="12.69140625" style="3" customWidth="1"/>
-    <col min="7426" max="7434" width="10.69140625" style="3" customWidth="1"/>
-    <col min="7435" max="7680" width="9.69140625" style="3"/>
-    <col min="7681" max="7681" width="12.69140625" style="3" customWidth="1"/>
-    <col min="7682" max="7690" width="10.69140625" style="3" customWidth="1"/>
-    <col min="7691" max="7936" width="9.69140625" style="3"/>
-    <col min="7937" max="7937" width="12.69140625" style="3" customWidth="1"/>
-    <col min="7938" max="7946" width="10.69140625" style="3" customWidth="1"/>
-    <col min="7947" max="8192" width="9.69140625" style="3"/>
-    <col min="8193" max="8193" width="12.69140625" style="3" customWidth="1"/>
-    <col min="8194" max="8202" width="10.69140625" style="3" customWidth="1"/>
-    <col min="8203" max="8448" width="9.69140625" style="3"/>
-    <col min="8449" max="8449" width="12.69140625" style="3" customWidth="1"/>
-    <col min="8450" max="8458" width="10.69140625" style="3" customWidth="1"/>
-    <col min="8459" max="8704" width="9.69140625" style="3"/>
-    <col min="8705" max="8705" width="12.69140625" style="3" customWidth="1"/>
-    <col min="8706" max="8714" width="10.69140625" style="3" customWidth="1"/>
-    <col min="8715" max="8960" width="9.69140625" style="3"/>
-    <col min="8961" max="8961" width="12.69140625" style="3" customWidth="1"/>
-    <col min="8962" max="8970" width="10.69140625" style="3" customWidth="1"/>
-    <col min="8971" max="9216" width="9.69140625" style="3"/>
-    <col min="9217" max="9217" width="12.69140625" style="3" customWidth="1"/>
-    <col min="9218" max="9226" width="10.69140625" style="3" customWidth="1"/>
-    <col min="9227" max="9472" width="9.69140625" style="3"/>
-    <col min="9473" max="9473" width="12.69140625" style="3" customWidth="1"/>
-    <col min="9474" max="9482" width="10.69140625" style="3" customWidth="1"/>
-    <col min="9483" max="9728" width="9.69140625" style="3"/>
-    <col min="9729" max="9729" width="12.69140625" style="3" customWidth="1"/>
-    <col min="9730" max="9738" width="10.69140625" style="3" customWidth="1"/>
-    <col min="9739" max="9984" width="9.69140625" style="3"/>
-    <col min="9985" max="9985" width="12.69140625" style="3" customWidth="1"/>
-    <col min="9986" max="9994" width="10.69140625" style="3" customWidth="1"/>
-    <col min="9995" max="10240" width="9.69140625" style="3"/>
-    <col min="10241" max="10241" width="12.69140625" style="3" customWidth="1"/>
-    <col min="10242" max="10250" width="10.69140625" style="3" customWidth="1"/>
-    <col min="10251" max="10496" width="9.69140625" style="3"/>
-    <col min="10497" max="10497" width="12.69140625" style="3" customWidth="1"/>
-    <col min="10498" max="10506" width="10.69140625" style="3" customWidth="1"/>
-    <col min="10507" max="10752" width="9.69140625" style="3"/>
-    <col min="10753" max="10753" width="12.69140625" style="3" customWidth="1"/>
-    <col min="10754" max="10762" width="10.69140625" style="3" customWidth="1"/>
-    <col min="10763" max="11008" width="9.69140625" style="3"/>
-    <col min="11009" max="11009" width="12.69140625" style="3" customWidth="1"/>
-    <col min="11010" max="11018" width="10.69140625" style="3" customWidth="1"/>
-    <col min="11019" max="11264" width="9.69140625" style="3"/>
-    <col min="11265" max="11265" width="12.69140625" style="3" customWidth="1"/>
-    <col min="11266" max="11274" width="10.69140625" style="3" customWidth="1"/>
-    <col min="11275" max="11520" width="9.69140625" style="3"/>
-    <col min="11521" max="11521" width="12.69140625" style="3" customWidth="1"/>
-    <col min="11522" max="11530" width="10.69140625" style="3" customWidth="1"/>
-    <col min="11531" max="11776" width="9.69140625" style="3"/>
-    <col min="11777" max="11777" width="12.69140625" style="3" customWidth="1"/>
-    <col min="11778" max="11786" width="10.69140625" style="3" customWidth="1"/>
-    <col min="11787" max="12032" width="9.69140625" style="3"/>
-    <col min="12033" max="12033" width="12.69140625" style="3" customWidth="1"/>
-    <col min="12034" max="12042" width="10.69140625" style="3" customWidth="1"/>
-    <col min="12043" max="12288" width="9.69140625" style="3"/>
-    <col min="12289" max="12289" width="12.69140625" style="3" customWidth="1"/>
-    <col min="12290" max="12298" width="10.69140625" style="3" customWidth="1"/>
-    <col min="12299" max="12544" width="9.69140625" style="3"/>
-    <col min="12545" max="12545" width="12.69140625" style="3" customWidth="1"/>
-    <col min="12546" max="12554" width="10.69140625" style="3" customWidth="1"/>
-    <col min="12555" max="12800" width="9.69140625" style="3"/>
-    <col min="12801" max="12801" width="12.69140625" style="3" customWidth="1"/>
-    <col min="12802" max="12810" width="10.69140625" style="3" customWidth="1"/>
-    <col min="12811" max="13056" width="9.69140625" style="3"/>
-    <col min="13057" max="13057" width="12.69140625" style="3" customWidth="1"/>
-    <col min="13058" max="13066" width="10.69140625" style="3" customWidth="1"/>
-    <col min="13067" max="13312" width="9.69140625" style="3"/>
-    <col min="13313" max="13313" width="12.69140625" style="3" customWidth="1"/>
-    <col min="13314" max="13322" width="10.69140625" style="3" customWidth="1"/>
-    <col min="13323" max="13568" width="9.69140625" style="3"/>
-    <col min="13569" max="13569" width="12.69140625" style="3" customWidth="1"/>
-    <col min="13570" max="13578" width="10.69140625" style="3" customWidth="1"/>
-    <col min="13579" max="13824" width="9.69140625" style="3"/>
-    <col min="13825" max="13825" width="12.69140625" style="3" customWidth="1"/>
-    <col min="13826" max="13834" width="10.69140625" style="3" customWidth="1"/>
-    <col min="13835" max="14080" width="9.69140625" style="3"/>
-    <col min="14081" max="14081" width="12.69140625" style="3" customWidth="1"/>
-    <col min="14082" max="14090" width="10.69140625" style="3" customWidth="1"/>
-    <col min="14091" max="14336" width="9.69140625" style="3"/>
-    <col min="14337" max="14337" width="12.69140625" style="3" customWidth="1"/>
-    <col min="14338" max="14346" width="10.69140625" style="3" customWidth="1"/>
-    <col min="14347" max="14592" width="9.69140625" style="3"/>
-    <col min="14593" max="14593" width="12.69140625" style="3" customWidth="1"/>
-    <col min="14594" max="14602" width="10.69140625" style="3" customWidth="1"/>
-    <col min="14603" max="14848" width="9.69140625" style="3"/>
-    <col min="14849" max="14849" width="12.69140625" style="3" customWidth="1"/>
-    <col min="14850" max="14858" width="10.69140625" style="3" customWidth="1"/>
-    <col min="14859" max="15104" width="9.69140625" style="3"/>
-    <col min="15105" max="15105" width="12.69140625" style="3" customWidth="1"/>
-    <col min="15106" max="15114" width="10.69140625" style="3" customWidth="1"/>
-    <col min="15115" max="15360" width="9.69140625" style="3"/>
-    <col min="15361" max="15361" width="12.69140625" style="3" customWidth="1"/>
-    <col min="15362" max="15370" width="10.69140625" style="3" customWidth="1"/>
-    <col min="15371" max="15616" width="9.69140625" style="3"/>
-    <col min="15617" max="15617" width="12.69140625" style="3" customWidth="1"/>
-    <col min="15618" max="15626" width="10.69140625" style="3" customWidth="1"/>
-    <col min="15627" max="15872" width="9.69140625" style="3"/>
-    <col min="15873" max="15873" width="12.69140625" style="3" customWidth="1"/>
-    <col min="15874" max="15882" width="10.69140625" style="3" customWidth="1"/>
-    <col min="15883" max="16128" width="9.69140625" style="3"/>
-    <col min="16129" max="16129" width="12.69140625" style="3" customWidth="1"/>
-    <col min="16130" max="16138" width="10.69140625" style="3" customWidth="1"/>
-    <col min="16139" max="16384" width="9.69140625" style="3"/>
+    <col min="1" max="1" width="12.6328125" style="2" customWidth="1"/>
+    <col min="2" max="10" width="10.6328125" style="2" customWidth="1"/>
+    <col min="11" max="256" width="9.6328125" style="3"/>
+    <col min="257" max="257" width="12.6328125" style="3" customWidth="1"/>
+    <col min="258" max="266" width="10.6328125" style="3" customWidth="1"/>
+    <col min="267" max="512" width="9.6328125" style="3"/>
+    <col min="513" max="513" width="12.6328125" style="3" customWidth="1"/>
+    <col min="514" max="522" width="10.6328125" style="3" customWidth="1"/>
+    <col min="523" max="768" width="9.6328125" style="3"/>
+    <col min="769" max="769" width="12.6328125" style="3" customWidth="1"/>
+    <col min="770" max="778" width="10.6328125" style="3" customWidth="1"/>
+    <col min="779" max="1024" width="9.6328125" style="3"/>
+    <col min="1025" max="1025" width="12.6328125" style="3" customWidth="1"/>
+    <col min="1026" max="1034" width="10.6328125" style="3" customWidth="1"/>
+    <col min="1035" max="1280" width="9.6328125" style="3"/>
+    <col min="1281" max="1281" width="12.6328125" style="3" customWidth="1"/>
+    <col min="1282" max="1290" width="10.6328125" style="3" customWidth="1"/>
+    <col min="1291" max="1536" width="9.6328125" style="3"/>
+    <col min="1537" max="1537" width="12.6328125" style="3" customWidth="1"/>
+    <col min="1538" max="1546" width="10.6328125" style="3" customWidth="1"/>
+    <col min="1547" max="1792" width="9.6328125" style="3"/>
+    <col min="1793" max="1793" width="12.6328125" style="3" customWidth="1"/>
+    <col min="1794" max="1802" width="10.6328125" style="3" customWidth="1"/>
+    <col min="1803" max="2048" width="9.6328125" style="3"/>
+    <col min="2049" max="2049" width="12.6328125" style="3" customWidth="1"/>
+    <col min="2050" max="2058" width="10.6328125" style="3" customWidth="1"/>
+    <col min="2059" max="2304" width="9.6328125" style="3"/>
+    <col min="2305" max="2305" width="12.6328125" style="3" customWidth="1"/>
+    <col min="2306" max="2314" width="10.6328125" style="3" customWidth="1"/>
+    <col min="2315" max="2560" width="9.6328125" style="3"/>
+    <col min="2561" max="2561" width="12.6328125" style="3" customWidth="1"/>
+    <col min="2562" max="2570" width="10.6328125" style="3" customWidth="1"/>
+    <col min="2571" max="2816" width="9.6328125" style="3"/>
+    <col min="2817" max="2817" width="12.6328125" style="3" customWidth="1"/>
+    <col min="2818" max="2826" width="10.6328125" style="3" customWidth="1"/>
+    <col min="2827" max="3072" width="9.6328125" style="3"/>
+    <col min="3073" max="3073" width="12.6328125" style="3" customWidth="1"/>
+    <col min="3074" max="3082" width="10.6328125" style="3" customWidth="1"/>
+    <col min="3083" max="3328" width="9.6328125" style="3"/>
+    <col min="3329" max="3329" width="12.6328125" style="3" customWidth="1"/>
+    <col min="3330" max="3338" width="10.6328125" style="3" customWidth="1"/>
+    <col min="3339" max="3584" width="9.6328125" style="3"/>
+    <col min="3585" max="3585" width="12.6328125" style="3" customWidth="1"/>
+    <col min="3586" max="3594" width="10.6328125" style="3" customWidth="1"/>
+    <col min="3595" max="3840" width="9.6328125" style="3"/>
+    <col min="3841" max="3841" width="12.6328125" style="3" customWidth="1"/>
+    <col min="3842" max="3850" width="10.6328125" style="3" customWidth="1"/>
+    <col min="3851" max="4096" width="9.6328125" style="3"/>
+    <col min="4097" max="4097" width="12.6328125" style="3" customWidth="1"/>
+    <col min="4098" max="4106" width="10.6328125" style="3" customWidth="1"/>
+    <col min="4107" max="4352" width="9.6328125" style="3"/>
+    <col min="4353" max="4353" width="12.6328125" style="3" customWidth="1"/>
+    <col min="4354" max="4362" width="10.6328125" style="3" customWidth="1"/>
+    <col min="4363" max="4608" width="9.6328125" style="3"/>
+    <col min="4609" max="4609" width="12.6328125" style="3" customWidth="1"/>
+    <col min="4610" max="4618" width="10.6328125" style="3" customWidth="1"/>
+    <col min="4619" max="4864" width="9.6328125" style="3"/>
+    <col min="4865" max="4865" width="12.6328125" style="3" customWidth="1"/>
+    <col min="4866" max="4874" width="10.6328125" style="3" customWidth="1"/>
+    <col min="4875" max="5120" width="9.6328125" style="3"/>
+    <col min="5121" max="5121" width="12.6328125" style="3" customWidth="1"/>
+    <col min="5122" max="5130" width="10.6328125" style="3" customWidth="1"/>
+    <col min="5131" max="5376" width="9.6328125" style="3"/>
+    <col min="5377" max="5377" width="12.6328125" style="3" customWidth="1"/>
+    <col min="5378" max="5386" width="10.6328125" style="3" customWidth="1"/>
+    <col min="5387" max="5632" width="9.6328125" style="3"/>
+    <col min="5633" max="5633" width="12.6328125" style="3" customWidth="1"/>
+    <col min="5634" max="5642" width="10.6328125" style="3" customWidth="1"/>
+    <col min="5643" max="5888" width="9.6328125" style="3"/>
+    <col min="5889" max="5889" width="12.6328125" style="3" customWidth="1"/>
+    <col min="5890" max="5898" width="10.6328125" style="3" customWidth="1"/>
+    <col min="5899" max="6144" width="9.6328125" style="3"/>
+    <col min="6145" max="6145" width="12.6328125" style="3" customWidth="1"/>
+    <col min="6146" max="6154" width="10.6328125" style="3" customWidth="1"/>
+    <col min="6155" max="6400" width="9.6328125" style="3"/>
+    <col min="6401" max="6401" width="12.6328125" style="3" customWidth="1"/>
+    <col min="6402" max="6410" width="10.6328125" style="3" customWidth="1"/>
+    <col min="6411" max="6656" width="9.6328125" style="3"/>
+    <col min="6657" max="6657" width="12.6328125" style="3" customWidth="1"/>
+    <col min="6658" max="6666" width="10.6328125" style="3" customWidth="1"/>
+    <col min="6667" max="6912" width="9.6328125" style="3"/>
+    <col min="6913" max="6913" width="12.6328125" style="3" customWidth="1"/>
+    <col min="6914" max="6922" width="10.6328125" style="3" customWidth="1"/>
+    <col min="6923" max="7168" width="9.6328125" style="3"/>
+    <col min="7169" max="7169" width="12.6328125" style="3" customWidth="1"/>
+    <col min="7170" max="7178" width="10.6328125" style="3" customWidth="1"/>
+    <col min="7179" max="7424" width="9.6328125" style="3"/>
+    <col min="7425" max="7425" width="12.6328125" style="3" customWidth="1"/>
+    <col min="7426" max="7434" width="10.6328125" style="3" customWidth="1"/>
+    <col min="7435" max="7680" width="9.6328125" style="3"/>
+    <col min="7681" max="7681" width="12.6328125" style="3" customWidth="1"/>
+    <col min="7682" max="7690" width="10.6328125" style="3" customWidth="1"/>
+    <col min="7691" max="7936" width="9.6328125" style="3"/>
+    <col min="7937" max="7937" width="12.6328125" style="3" customWidth="1"/>
+    <col min="7938" max="7946" width="10.6328125" style="3" customWidth="1"/>
+    <col min="7947" max="8192" width="9.6328125" style="3"/>
+    <col min="8193" max="8193" width="12.6328125" style="3" customWidth="1"/>
+    <col min="8194" max="8202" width="10.6328125" style="3" customWidth="1"/>
+    <col min="8203" max="8448" width="9.6328125" style="3"/>
+    <col min="8449" max="8449" width="12.6328125" style="3" customWidth="1"/>
+    <col min="8450" max="8458" width="10.6328125" style="3" customWidth="1"/>
+    <col min="8459" max="8704" width="9.6328125" style="3"/>
+    <col min="8705" max="8705" width="12.6328125" style="3" customWidth="1"/>
+    <col min="8706" max="8714" width="10.6328125" style="3" customWidth="1"/>
+    <col min="8715" max="8960" width="9.6328125" style="3"/>
+    <col min="8961" max="8961" width="12.6328125" style="3" customWidth="1"/>
+    <col min="8962" max="8970" width="10.6328125" style="3" customWidth="1"/>
+    <col min="8971" max="9216" width="9.6328125" style="3"/>
+    <col min="9217" max="9217" width="12.6328125" style="3" customWidth="1"/>
+    <col min="9218" max="9226" width="10.6328125" style="3" customWidth="1"/>
+    <col min="9227" max="9472" width="9.6328125" style="3"/>
+    <col min="9473" max="9473" width="12.6328125" style="3" customWidth="1"/>
+    <col min="9474" max="9482" width="10.6328125" style="3" customWidth="1"/>
+    <col min="9483" max="9728" width="9.6328125" style="3"/>
+    <col min="9729" max="9729" width="12.6328125" style="3" customWidth="1"/>
+    <col min="9730" max="9738" width="10.6328125" style="3" customWidth="1"/>
+    <col min="9739" max="9984" width="9.6328125" style="3"/>
+    <col min="9985" max="9985" width="12.6328125" style="3" customWidth="1"/>
+    <col min="9986" max="9994" width="10.6328125" style="3" customWidth="1"/>
+    <col min="9995" max="10240" width="9.6328125" style="3"/>
+    <col min="10241" max="10241" width="12.6328125" style="3" customWidth="1"/>
+    <col min="10242" max="10250" width="10.6328125" style="3" customWidth="1"/>
+    <col min="10251" max="10496" width="9.6328125" style="3"/>
+    <col min="10497" max="10497" width="12.6328125" style="3" customWidth="1"/>
+    <col min="10498" max="10506" width="10.6328125" style="3" customWidth="1"/>
+    <col min="10507" max="10752" width="9.6328125" style="3"/>
+    <col min="10753" max="10753" width="12.6328125" style="3" customWidth="1"/>
+    <col min="10754" max="10762" width="10.6328125" style="3" customWidth="1"/>
+    <col min="10763" max="11008" width="9.6328125" style="3"/>
+    <col min="11009" max="11009" width="12.6328125" style="3" customWidth="1"/>
+    <col min="11010" max="11018" width="10.6328125" style="3" customWidth="1"/>
+    <col min="11019" max="11264" width="9.6328125" style="3"/>
+    <col min="11265" max="11265" width="12.6328125" style="3" customWidth="1"/>
+    <col min="11266" max="11274" width="10.6328125" style="3" customWidth="1"/>
+    <col min="11275" max="11520" width="9.6328125" style="3"/>
+    <col min="11521" max="11521" width="12.6328125" style="3" customWidth="1"/>
+    <col min="11522" max="11530" width="10.6328125" style="3" customWidth="1"/>
+    <col min="11531" max="11776" width="9.6328125" style="3"/>
+    <col min="11777" max="11777" width="12.6328125" style="3" customWidth="1"/>
+    <col min="11778" max="11786" width="10.6328125" style="3" customWidth="1"/>
+    <col min="11787" max="12032" width="9.6328125" style="3"/>
+    <col min="12033" max="12033" width="12.6328125" style="3" customWidth="1"/>
+    <col min="12034" max="12042" width="10.6328125" style="3" customWidth="1"/>
+    <col min="12043" max="12288" width="9.6328125" style="3"/>
+    <col min="12289" max="12289" width="12.6328125" style="3" customWidth="1"/>
+    <col min="12290" max="12298" width="10.6328125" style="3" customWidth="1"/>
+    <col min="12299" max="12544" width="9.6328125" style="3"/>
+    <col min="12545" max="12545" width="12.6328125" style="3" customWidth="1"/>
+    <col min="12546" max="12554" width="10.6328125" style="3" customWidth="1"/>
+    <col min="12555" max="12800" width="9.6328125" style="3"/>
+    <col min="12801" max="12801" width="12.6328125" style="3" customWidth="1"/>
+    <col min="12802" max="12810" width="10.6328125" style="3" customWidth="1"/>
+    <col min="12811" max="13056" width="9.6328125" style="3"/>
+    <col min="13057" max="13057" width="12.6328125" style="3" customWidth="1"/>
+    <col min="13058" max="13066" width="10.6328125" style="3" customWidth="1"/>
+    <col min="13067" max="13312" width="9.6328125" style="3"/>
+    <col min="13313" max="13313" width="12.6328125" style="3" customWidth="1"/>
+    <col min="13314" max="13322" width="10.6328125" style="3" customWidth="1"/>
+    <col min="13323" max="13568" width="9.6328125" style="3"/>
+    <col min="13569" max="13569" width="12.6328125" style="3" customWidth="1"/>
+    <col min="13570" max="13578" width="10.6328125" style="3" customWidth="1"/>
+    <col min="13579" max="13824" width="9.6328125" style="3"/>
+    <col min="13825" max="13825" width="12.6328125" style="3" customWidth="1"/>
+    <col min="13826" max="13834" width="10.6328125" style="3" customWidth="1"/>
+    <col min="13835" max="14080" width="9.6328125" style="3"/>
+    <col min="14081" max="14081" width="12.6328125" style="3" customWidth="1"/>
+    <col min="14082" max="14090" width="10.6328125" style="3" customWidth="1"/>
+    <col min="14091" max="14336" width="9.6328125" style="3"/>
+    <col min="14337" max="14337" width="12.6328125" style="3" customWidth="1"/>
+    <col min="14338" max="14346" width="10.6328125" style="3" customWidth="1"/>
+    <col min="14347" max="14592" width="9.6328125" style="3"/>
+    <col min="14593" max="14593" width="12.6328125" style="3" customWidth="1"/>
+    <col min="14594" max="14602" width="10.6328125" style="3" customWidth="1"/>
+    <col min="14603" max="14848" width="9.6328125" style="3"/>
+    <col min="14849" max="14849" width="12.6328125" style="3" customWidth="1"/>
+    <col min="14850" max="14858" width="10.6328125" style="3" customWidth="1"/>
+    <col min="14859" max="15104" width="9.6328125" style="3"/>
+    <col min="15105" max="15105" width="12.6328125" style="3" customWidth="1"/>
+    <col min="15106" max="15114" width="10.6328125" style="3" customWidth="1"/>
+    <col min="15115" max="15360" width="9.6328125" style="3"/>
+    <col min="15361" max="15361" width="12.6328125" style="3" customWidth="1"/>
+    <col min="15362" max="15370" width="10.6328125" style="3" customWidth="1"/>
+    <col min="15371" max="15616" width="9.6328125" style="3"/>
+    <col min="15617" max="15617" width="12.6328125" style="3" customWidth="1"/>
+    <col min="15618" max="15626" width="10.6328125" style="3" customWidth="1"/>
+    <col min="15627" max="15872" width="9.6328125" style="3"/>
+    <col min="15873" max="15873" width="12.6328125" style="3" customWidth="1"/>
+    <col min="15874" max="15882" width="10.6328125" style="3" customWidth="1"/>
+    <col min="15883" max="16128" width="9.6328125" style="3"/>
+    <col min="16129" max="16129" width="12.6328125" style="3" customWidth="1"/>
+    <col min="16130" max="16138" width="10.6328125" style="3" customWidth="1"/>
+    <col min="16139" max="16384" width="9.6328125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="J1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="25.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -57136,7 +57161,7 @@
       <c r="I2" s="5"/>
       <c r="J2" s="6"/>
     </row>
-    <row r="3" spans="1:10" s="9" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:10" s="9" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
@@ -57150,7 +57175,7 @@
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
     </row>
-    <row r="4" spans="1:10" ht="20.149999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:10" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>3</v>
       </c>
@@ -57164,7 +57189,7 @@
       <c r="I4" s="11"/>
       <c r="J4" s="11"/>
     </row>
-    <row r="5" spans="1:10" ht="25.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="25.35" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>4</v>
       </c>
@@ -57177,1640 +57202,1711 @@
         <v>6</v>
       </c>
       <c r="F5" s="13"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="17" t="s">
+      <c r="G5" s="14"/>
+      <c r="H5" s="15" t="s">
         <v>7</v>
       </c>
       <c r="I5" s="13"/>
       <c r="J5" s="13"/>
     </row>
-    <row r="6" spans="1:10" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="18"/>
-      <c r="B6" s="19" t="s">
+    <row r="6" spans="1:10" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="16"/>
+      <c r="B6" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="22" t="s">
+      <c r="G6" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="23" t="s">
+      <c r="H6" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="I6" s="19" t="s">
+      <c r="I6" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="J6" s="19" t="s">
+      <c r="J6" s="17" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="30.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="24" t="s">
+    <row r="7" spans="1:10" ht="30.6" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="29"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="26"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="22"/>
     </row>
-    <row r="8" spans="1:10" ht="25.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="30" t="s">
+    <row r="8" spans="1:10" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="31">
-        <v>-774205</v>
-      </c>
-      <c r="C8" s="31">
-        <v>-1057495</v>
-      </c>
-      <c r="D8" s="32">
-        <v>283290</v>
-      </c>
-      <c r="E8" s="33">
-        <v>3092536</v>
-      </c>
-      <c r="F8" s="31">
-        <v>2047457</v>
-      </c>
-      <c r="G8" s="34">
-        <v>1045079</v>
-      </c>
-      <c r="H8" s="35">
-        <v>3866741</v>
-      </c>
-      <c r="I8" s="31">
-        <v>3104952</v>
-      </c>
-      <c r="J8" s="32">
-        <v>761789</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="36" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="37">
-        <v>-68800</v>
-      </c>
-      <c r="C9" s="37">
-        <v>-91071</v>
-      </c>
-      <c r="D9" s="38">
-        <v>22271</v>
-      </c>
-      <c r="E9" s="39">
-        <v>259974</v>
-      </c>
-      <c r="F9" s="37">
-        <v>175518</v>
-      </c>
-      <c r="G9" s="40">
-        <v>84456</v>
-      </c>
-      <c r="H9" s="41">
-        <v>328774</v>
-      </c>
-      <c r="I9" s="37">
-        <v>266589</v>
-      </c>
-      <c r="J9" s="38">
-        <v>62185</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="36" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="37">
-        <v>-69202</v>
-      </c>
-      <c r="C10" s="37">
-        <v>-92171</v>
-      </c>
-      <c r="D10" s="38">
-        <v>22969</v>
-      </c>
-      <c r="E10" s="39">
-        <v>254337</v>
-      </c>
-      <c r="F10" s="37">
-        <v>169282</v>
-      </c>
-      <c r="G10" s="40">
-        <v>85055</v>
-      </c>
-      <c r="H10" s="41">
-        <v>323539</v>
-      </c>
-      <c r="I10" s="37">
-        <v>261453</v>
-      </c>
-      <c r="J10" s="38">
-        <v>62086</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="36" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="37">
-        <v>-58587</v>
-      </c>
-      <c r="C11" s="37">
-        <v>-81937</v>
-      </c>
-      <c r="D11" s="38">
-        <v>23351</v>
-      </c>
-      <c r="E11" s="39">
-        <v>259541</v>
-      </c>
-      <c r="F11" s="37">
-        <v>174112</v>
-      </c>
-      <c r="G11" s="40">
-        <v>85429</v>
-      </c>
-      <c r="H11" s="41">
-        <v>318127</v>
-      </c>
-      <c r="I11" s="37">
-        <v>256049</v>
-      </c>
-      <c r="J11" s="38">
-        <v>62079</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="36" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="37">
-        <v>-71110</v>
-      </c>
-      <c r="C12" s="37">
-        <v>-93950</v>
-      </c>
-      <c r="D12" s="38">
-        <v>22840</v>
-      </c>
-      <c r="E12" s="39">
-        <v>253608</v>
-      </c>
-      <c r="F12" s="37">
-        <v>167547</v>
-      </c>
-      <c r="G12" s="40">
-        <v>86061</v>
-      </c>
-      <c r="H12" s="41">
-        <v>324718</v>
-      </c>
-      <c r="I12" s="37">
-        <v>261497</v>
-      </c>
-      <c r="J12" s="38">
-        <v>63222</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="36" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="37">
-        <v>-65814</v>
-      </c>
-      <c r="C13" s="37">
-        <v>-89397</v>
-      </c>
-      <c r="D13" s="38">
-        <v>23584</v>
-      </c>
-      <c r="E13" s="39">
-        <v>252569</v>
-      </c>
-      <c r="F13" s="37">
-        <v>165994</v>
-      </c>
-      <c r="G13" s="40">
-        <v>86575</v>
-      </c>
-      <c r="H13" s="41">
-        <v>318383</v>
-      </c>
-      <c r="I13" s="37">
-        <v>255391</v>
-      </c>
-      <c r="J13" s="38">
-        <v>62992</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="36" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="37">
-        <v>-65163</v>
-      </c>
-      <c r="C14" s="37">
-        <v>-88851</v>
-      </c>
-      <c r="D14" s="38">
-        <v>23688</v>
-      </c>
-      <c r="E14" s="39">
-        <v>251879</v>
-      </c>
-      <c r="F14" s="37">
-        <v>164797</v>
-      </c>
-      <c r="G14" s="40">
-        <v>87082</v>
-      </c>
-      <c r="H14" s="41">
-        <v>317042</v>
-      </c>
-      <c r="I14" s="37">
-        <v>253648</v>
-      </c>
-      <c r="J14" s="38">
-        <v>63394</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="37">
-        <v>-63759</v>
-      </c>
-      <c r="C15" s="37">
-        <v>-88294</v>
-      </c>
-      <c r="D15" s="38">
-        <v>24535</v>
-      </c>
-      <c r="E15" s="39">
-        <v>255576</v>
-      </c>
-      <c r="F15" s="37">
-        <v>168286</v>
-      </c>
-      <c r="G15" s="40">
-        <v>87290</v>
-      </c>
-      <c r="H15" s="41">
-        <v>319335</v>
-      </c>
-      <c r="I15" s="37">
-        <v>256580</v>
-      </c>
-      <c r="J15" s="38">
-        <v>62755</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="36" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="37">
-        <v>-59165</v>
-      </c>
-      <c r="C16" s="37">
-        <v>-84221</v>
-      </c>
-      <c r="D16" s="38">
-        <v>25055</v>
-      </c>
-      <c r="E16" s="39">
-        <v>259963</v>
-      </c>
-      <c r="F16" s="37">
-        <v>172138</v>
-      </c>
-      <c r="G16" s="40">
-        <v>87825</v>
-      </c>
-      <c r="H16" s="41">
-        <v>319128</v>
-      </c>
-      <c r="I16" s="37">
-        <v>256358</v>
-      </c>
-      <c r="J16" s="38">
-        <v>62770</v>
-      </c>
-    </row>
-    <row r="17" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="37">
-        <v>-59565</v>
-      </c>
-      <c r="C17" s="37">
-        <v>-83759</v>
-      </c>
-      <c r="D17" s="38">
-        <v>24194</v>
-      </c>
-      <c r="E17" s="39">
-        <v>263533</v>
-      </c>
-      <c r="F17" s="37">
-        <v>175342</v>
-      </c>
-      <c r="G17" s="40">
-        <v>88191</v>
-      </c>
-      <c r="H17" s="41">
-        <v>323098</v>
-      </c>
-      <c r="I17" s="37">
-        <v>259101</v>
-      </c>
-      <c r="J17" s="38">
-        <v>63997</v>
-      </c>
-    </row>
-    <row r="18" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="36" t="s">
-        <v>22</v>
-      </c>
-      <c r="B18" s="37">
-        <v>-64100</v>
-      </c>
-      <c r="C18" s="37">
-        <v>-87230</v>
-      </c>
-      <c r="D18" s="38">
-        <v>23130</v>
-      </c>
-      <c r="E18" s="39">
-        <v>262463</v>
-      </c>
-      <c r="F18" s="37">
-        <v>174325</v>
-      </c>
-      <c r="G18" s="40">
-        <v>88138</v>
-      </c>
-      <c r="H18" s="41">
-        <v>326563</v>
-      </c>
-      <c r="I18" s="37">
-        <v>261555</v>
-      </c>
-      <c r="J18" s="38">
-        <v>65008</v>
-      </c>
-    </row>
-    <row r="19" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="36" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="37">
-        <v>-65053</v>
-      </c>
-      <c r="C19" s="37">
-        <v>-88444</v>
-      </c>
-      <c r="D19" s="38">
-        <v>23391</v>
-      </c>
-      <c r="E19" s="39">
-        <v>257254</v>
-      </c>
-      <c r="F19" s="37">
-        <v>168469</v>
-      </c>
-      <c r="G19" s="40">
-        <v>88785</v>
-      </c>
-      <c r="H19" s="41">
-        <v>322307</v>
-      </c>
-      <c r="I19" s="37">
-        <v>256913</v>
-      </c>
-      <c r="J19" s="38">
-        <v>65394</v>
-      </c>
-    </row>
-    <row r="20" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="36" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" s="37">
-        <v>-63888</v>
-      </c>
-      <c r="C20" s="37">
-        <v>-88171</v>
-      </c>
-      <c r="D20" s="38">
-        <v>24284</v>
-      </c>
-      <c r="E20" s="39">
-        <v>261838</v>
-      </c>
-      <c r="F20" s="37">
-        <v>171647</v>
-      </c>
-      <c r="G20" s="40">
-        <v>90191</v>
-      </c>
-      <c r="H20" s="41">
-        <v>325726</v>
-      </c>
-      <c r="I20" s="37">
-        <v>259819</v>
-      </c>
-      <c r="J20" s="38">
-        <v>65907</v>
-      </c>
-      <c r="K20" s="42"/>
-      <c r="L20" s="42"/>
-      <c r="M20" s="42"/>
-      <c r="N20" s="42"/>
-      <c r="O20" s="42"/>
-      <c r="P20" s="42"/>
-      <c r="Q20" s="42"/>
-      <c r="R20" s="42"/>
-      <c r="S20" s="42"/>
-      <c r="T20" s="42"/>
-      <c r="U20" s="42"/>
-      <c r="V20" s="42"/>
-      <c r="W20" s="42"/>
-      <c r="X20" s="42"/>
-      <c r="Y20" s="42"/>
-      <c r="Z20" s="42"/>
-      <c r="AA20" s="42"/>
-      <c r="AB20" s="42"/>
-      <c r="AC20" s="42"/>
-      <c r="AD20" s="42"/>
-      <c r="AE20" s="42"/>
-      <c r="AF20" s="42"/>
-      <c r="AG20" s="42"/>
-      <c r="AH20" s="42"/>
-      <c r="AI20" s="42"/>
-      <c r="AJ20" s="42"/>
-      <c r="AK20" s="42"/>
-      <c r="AL20" s="42"/>
-      <c r="AM20" s="42"/>
-      <c r="AN20" s="42"/>
-      <c r="AO20" s="42"/>
-      <c r="AP20" s="42"/>
-      <c r="AQ20" s="42"/>
-      <c r="AR20" s="42"/>
-      <c r="AS20" s="42"/>
-      <c r="AT20" s="42"/>
-      <c r="AU20" s="42"/>
-      <c r="AV20" s="42"/>
-      <c r="AW20" s="42"/>
-      <c r="AX20" s="42"/>
-      <c r="AY20" s="42"/>
-      <c r="AZ20" s="42"/>
-      <c r="BA20" s="42"/>
-      <c r="BB20" s="42"/>
-      <c r="BC20" s="42"/>
-      <c r="BD20" s="42"/>
-      <c r="BE20" s="42"/>
-      <c r="BF20" s="42"/>
-      <c r="BG20" s="42"/>
-      <c r="BH20" s="42"/>
-      <c r="BI20" s="42"/>
-      <c r="BJ20" s="42"/>
-      <c r="BK20" s="42"/>
-      <c r="BL20" s="42"/>
-      <c r="BM20" s="42"/>
-      <c r="BN20" s="42"/>
-      <c r="BO20" s="42"/>
-      <c r="BP20" s="42"/>
-      <c r="BQ20" s="42"/>
-      <c r="BR20" s="42"/>
-      <c r="BS20" s="42"/>
-      <c r="BT20" s="42"/>
-      <c r="BU20" s="42"/>
-      <c r="BV20" s="42"/>
-      <c r="BW20" s="42"/>
-      <c r="BX20" s="42"/>
-      <c r="BY20" s="42"/>
-      <c r="BZ20" s="42"/>
-      <c r="CA20" s="42"/>
-      <c r="CB20" s="42"/>
-      <c r="CC20" s="42"/>
-      <c r="CD20" s="42"/>
-      <c r="CE20" s="42"/>
-      <c r="CF20" s="42"/>
-      <c r="CG20" s="42"/>
-      <c r="CH20" s="42"/>
-      <c r="CI20" s="42"/>
-      <c r="CJ20" s="42"/>
-      <c r="CK20" s="42"/>
-      <c r="CL20" s="42"/>
-      <c r="CM20" s="42"/>
-      <c r="CN20" s="42"/>
-      <c r="CO20" s="42"/>
-      <c r="CP20" s="42"/>
-      <c r="CQ20" s="42"/>
-      <c r="CR20" s="42"/>
-      <c r="CS20" s="42"/>
-      <c r="CT20" s="42"/>
-      <c r="CU20" s="42"/>
-      <c r="CV20" s="42"/>
-      <c r="CW20" s="42"/>
-      <c r="CX20" s="42"/>
-      <c r="CY20" s="42"/>
-      <c r="CZ20" s="42"/>
-      <c r="DA20" s="42"/>
-      <c r="DB20" s="42"/>
-      <c r="DC20" s="42"/>
-      <c r="DD20" s="42"/>
-      <c r="DE20" s="42"/>
-      <c r="DF20" s="42"/>
-      <c r="DG20" s="42"/>
-      <c r="DH20" s="42"/>
-      <c r="DI20" s="42"/>
-      <c r="DJ20" s="42"/>
-      <c r="DK20" s="42"/>
-      <c r="DL20" s="42"/>
-      <c r="DM20" s="42"/>
-      <c r="DN20" s="42"/>
-      <c r="DO20" s="42"/>
-      <c r="DP20" s="42"/>
-      <c r="DQ20" s="42"/>
-      <c r="DR20" s="42"/>
-      <c r="DS20" s="42"/>
-      <c r="DT20" s="42"/>
-      <c r="DU20" s="42"/>
-      <c r="DV20" s="42"/>
-      <c r="DW20" s="42"/>
-      <c r="DX20" s="42"/>
-      <c r="DY20" s="42"/>
-      <c r="DZ20" s="42"/>
-      <c r="EA20" s="42"/>
-      <c r="EB20" s="42"/>
-      <c r="EC20" s="42"/>
-      <c r="ED20" s="42"/>
-      <c r="EE20" s="42"/>
-      <c r="EF20" s="42"/>
-      <c r="EG20" s="42"/>
-      <c r="EH20" s="42"/>
-      <c r="EI20" s="42"/>
-      <c r="EJ20" s="42"/>
-      <c r="EK20" s="42"/>
-      <c r="EL20" s="42"/>
-      <c r="EM20" s="42"/>
-      <c r="EN20" s="42"/>
-      <c r="EO20" s="42"/>
-      <c r="EP20" s="42"/>
-      <c r="EQ20" s="42"/>
-      <c r="ER20" s="42"/>
-      <c r="ES20" s="42"/>
-      <c r="ET20" s="42"/>
-      <c r="EU20" s="42"/>
-      <c r="EV20" s="42"/>
-      <c r="EW20" s="42"/>
-      <c r="EX20" s="42"/>
-      <c r="EY20" s="42"/>
-      <c r="EZ20" s="42"/>
-      <c r="FA20" s="42"/>
-      <c r="FB20" s="42"/>
-      <c r="FC20" s="42"/>
-      <c r="FD20" s="42"/>
-      <c r="FE20" s="42"/>
-      <c r="FF20" s="42"/>
-      <c r="FG20" s="42"/>
-      <c r="FH20" s="42"/>
-      <c r="FI20" s="42"/>
-      <c r="FJ20" s="42"/>
-      <c r="FK20" s="42"/>
-      <c r="FL20" s="42"/>
-      <c r="FM20" s="42"/>
-      <c r="FN20" s="42"/>
-      <c r="FO20" s="42"/>
-      <c r="FP20" s="42"/>
-      <c r="FQ20" s="42"/>
-      <c r="FR20" s="42"/>
-      <c r="FS20" s="42"/>
-      <c r="FT20" s="42"/>
-      <c r="FU20" s="42"/>
-      <c r="FV20" s="42"/>
-      <c r="FW20" s="42"/>
-      <c r="FX20" s="42"/>
-      <c r="FY20" s="42"/>
-      <c r="FZ20" s="42"/>
-      <c r="GA20" s="42"/>
-      <c r="GB20" s="42"/>
-      <c r="GC20" s="42"/>
-      <c r="GD20" s="42"/>
-      <c r="GE20" s="42"/>
-      <c r="GF20" s="42"/>
-      <c r="GG20" s="42"/>
-      <c r="GH20" s="42"/>
-      <c r="GI20" s="42"/>
-      <c r="GJ20" s="42"/>
-      <c r="GK20" s="42"/>
-      <c r="GL20" s="42"/>
-      <c r="GM20" s="42"/>
-      <c r="GN20" s="42"/>
-      <c r="GO20" s="42"/>
-      <c r="GP20" s="42"/>
-      <c r="GQ20" s="42"/>
-      <c r="GR20" s="42"/>
-      <c r="GS20" s="42"/>
-      <c r="GT20" s="42"/>
-      <c r="GU20" s="42"/>
-      <c r="GV20" s="42"/>
-      <c r="GW20" s="42"/>
-      <c r="GX20" s="42"/>
-      <c r="GY20" s="42"/>
-      <c r="GZ20" s="42"/>
-      <c r="HA20" s="42"/>
-      <c r="HB20" s="42"/>
-      <c r="HC20" s="42"/>
-      <c r="HD20" s="42"/>
-      <c r="HE20" s="42"/>
-      <c r="HF20" s="42"/>
-      <c r="HG20" s="42"/>
-      <c r="HH20" s="42"/>
-      <c r="HI20" s="42"/>
-      <c r="HJ20" s="42"/>
-      <c r="HK20" s="42"/>
-      <c r="HL20" s="42"/>
-      <c r="HM20" s="42"/>
-      <c r="HN20" s="42"/>
-      <c r="HO20" s="42"/>
-      <c r="HP20" s="42"/>
-      <c r="HQ20" s="42"/>
-      <c r="HR20" s="42"/>
-      <c r="HS20" s="42"/>
-      <c r="HT20" s="42"/>
-      <c r="HU20" s="42"/>
-      <c r="HV20" s="42"/>
-      <c r="HW20" s="42"/>
-      <c r="HX20" s="42"/>
-      <c r="HY20" s="42"/>
-    </row>
-    <row r="21" spans="1:233" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="43" t="s">
-        <v>25</v>
-      </c>
-      <c r="B21" s="44"/>
-      <c r="C21" s="44"/>
-      <c r="D21" s="45"/>
-      <c r="E21" s="46"/>
-      <c r="F21" s="44"/>
-      <c r="G21" s="47"/>
-      <c r="H21" s="48"/>
-      <c r="I21" s="44"/>
-      <c r="J21" s="45"/>
-    </row>
-    <row r="22" spans="1:233" ht="25.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="30" t="s">
-        <v>12</v>
-      </c>
-      <c r="B22" s="31">
+      <c r="B8" s="27">
         <v>-903532</v>
       </c>
-      <c r="C22" s="31">
+      <c r="C8" s="27">
         <v>-1215403</v>
       </c>
-      <c r="D22" s="32">
+      <c r="D8" s="28">
         <v>311870</v>
       </c>
-      <c r="E22" s="33">
+      <c r="E8" s="29">
         <v>3232524</v>
       </c>
-      <c r="F22" s="31">
+      <c r="F8" s="27">
         <v>2079777</v>
       </c>
-      <c r="G22" s="34">
+      <c r="G8" s="30">
         <v>1152747</v>
       </c>
-      <c r="H22" s="35">
+      <c r="H8" s="31">
         <v>4136057</v>
       </c>
-      <c r="I22" s="31">
+      <c r="I8" s="27">
         <v>3295180</v>
       </c>
-      <c r="J22" s="32">
+      <c r="J8" s="28">
         <v>840877</v>
       </c>
     </row>
-    <row r="23" spans="1:233" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="36" t="s">
+    <row r="9" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="37">
+      <c r="B9" s="33">
         <v>-67077</v>
       </c>
-      <c r="C23" s="37">
+      <c r="C9" s="33">
         <v>-92640</v>
       </c>
-      <c r="D23" s="38">
+      <c r="D9" s="34">
         <v>25562</v>
       </c>
-      <c r="E23" s="39">
+      <c r="E9" s="35">
         <v>261796</v>
       </c>
-      <c r="F23" s="37">
+      <c r="F9" s="33">
         <v>170216</v>
       </c>
-      <c r="G23" s="40">
+      <c r="G9" s="36">
         <v>91579</v>
       </c>
-      <c r="H23" s="41">
+      <c r="H9" s="37">
         <v>328873</v>
       </c>
-      <c r="I23" s="37">
+      <c r="I9" s="33">
         <v>262856</v>
       </c>
-      <c r="J23" s="38">
+      <c r="J9" s="34">
         <v>66017</v>
       </c>
     </row>
-    <row r="24" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="36" t="s">
+    <row r="10" spans="1:10" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B24" s="37">
+      <c r="B10" s="27">
+        <v>-67077</v>
+      </c>
+      <c r="C10" s="27">
+        <v>-92640</v>
+      </c>
+      <c r="D10" s="28">
+        <v>25562</v>
+      </c>
+      <c r="E10" s="29">
+        <v>261796</v>
+      </c>
+      <c r="F10" s="27">
+        <v>170216</v>
+      </c>
+      <c r="G10" s="30">
+        <v>91579</v>
+      </c>
+      <c r="H10" s="31">
+        <v>328873</v>
+      </c>
+      <c r="I10" s="27">
+        <v>262856</v>
+      </c>
+      <c r="J10" s="28">
+        <v>66017</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="27">
         <v>-66431</v>
       </c>
-      <c r="C24" s="37">
+      <c r="C11" s="27">
         <v>-92390</v>
       </c>
-      <c r="D24" s="38">
+      <c r="D11" s="28">
         <v>25959</v>
       </c>
-      <c r="E24" s="39">
+      <c r="E11" s="29">
         <v>269323</v>
       </c>
-      <c r="F24" s="37">
+      <c r="F11" s="27">
         <v>175344</v>
       </c>
-      <c r="G24" s="40">
+      <c r="G11" s="30">
         <v>93979</v>
       </c>
-      <c r="H24" s="41">
+      <c r="H11" s="31">
         <v>335754</v>
       </c>
-      <c r="I24" s="37">
+      <c r="I11" s="27">
         <v>267734</v>
       </c>
-      <c r="J24" s="38">
+      <c r="J11" s="28">
         <v>68021</v>
       </c>
     </row>
-    <row r="25" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="36" t="s">
-        <v>15</v>
+    <row r="12" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="26" t="s">
+        <v>16</v>
       </c>
-      <c r="B25" s="37">
+      <c r="B12" s="27">
         <v>-66266</v>
       </c>
-      <c r="C25" s="37">
+      <c r="C12" s="27">
         <v>-93122</v>
       </c>
-      <c r="D25" s="38">
+      <c r="D12" s="28">
         <v>26857</v>
       </c>
-      <c r="E25" s="39">
+      <c r="E12" s="29">
         <v>265638</v>
       </c>
-      <c r="F25" s="37">
+      <c r="F12" s="27">
         <v>171506</v>
       </c>
-      <c r="G25" s="40">
+      <c r="G12" s="30">
         <v>94131</v>
       </c>
-      <c r="H25" s="41">
+      <c r="H12" s="31">
         <v>331904</v>
       </c>
-      <c r="I25" s="37">
+      <c r="I12" s="27">
         <v>264629</v>
       </c>
-      <c r="J25" s="38">
+      <c r="J12" s="28">
         <v>67275</v>
       </c>
     </row>
-    <row r="26" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="36" t="s">
-        <v>16</v>
+    <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="26" t="s">
+        <v>17</v>
       </c>
-      <c r="B26" s="37">
+      <c r="B13" s="27">
         <v>-73110</v>
       </c>
-      <c r="C26" s="37">
+      <c r="C13" s="27">
         <v>-98957</v>
       </c>
-      <c r="D26" s="38">
+      <c r="D13" s="28">
         <v>25847</v>
       </c>
-      <c r="E26" s="39">
+      <c r="E13" s="29">
         <v>266393</v>
       </c>
-      <c r="F26" s="37">
+      <c r="F13" s="27">
         <v>173037</v>
       </c>
-      <c r="G26" s="40">
+      <c r="G13" s="30">
         <v>93356</v>
       </c>
-      <c r="H26" s="41">
+      <c r="H13" s="31">
         <v>339503</v>
       </c>
-      <c r="I26" s="37">
+      <c r="I13" s="27">
         <v>271994</v>
       </c>
-      <c r="J26" s="38">
+      <c r="J13" s="28">
         <v>67509</v>
       </c>
     </row>
-    <row r="27" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="36" t="s">
-        <v>17</v>
+    <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="26" t="s">
+        <v>18</v>
       </c>
-      <c r="B27" s="37">
+      <c r="B14" s="27">
         <v>-74456</v>
       </c>
-      <c r="C27" s="37">
+      <c r="C14" s="27">
         <v>-100630</v>
       </c>
-      <c r="D27" s="38">
+      <c r="D14" s="28">
         <v>26174</v>
       </c>
-      <c r="E27" s="39">
+      <c r="E14" s="29">
         <v>264976</v>
       </c>
-      <c r="F27" s="37">
+      <c r="F14" s="27">
         <v>170321</v>
       </c>
-      <c r="G27" s="40">
+      <c r="G14" s="30">
         <v>94655</v>
       </c>
-      <c r="H27" s="41">
+      <c r="H14" s="31">
         <v>339432</v>
       </c>
-      <c r="I27" s="37">
+      <c r="I14" s="27">
         <v>270951</v>
       </c>
-      <c r="J27" s="38">
+      <c r="J14" s="28">
         <v>68481</v>
       </c>
     </row>
-    <row r="28" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="36" t="s">
-        <v>18</v>
+    <row r="15" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="26" t="s">
+        <v>19</v>
       </c>
-      <c r="B28" s="37">
+      <c r="B15" s="27">
         <v>-73892</v>
       </c>
-      <c r="C28" s="37">
+      <c r="C15" s="27">
         <v>-99563</v>
       </c>
-      <c r="D28" s="38">
+      <c r="D15" s="28">
         <v>25671</v>
       </c>
-      <c r="E28" s="39">
+      <c r="E15" s="29">
         <v>268356</v>
       </c>
-      <c r="F28" s="37">
+      <c r="F15" s="27">
         <v>173318</v>
       </c>
-      <c r="G28" s="40">
+      <c r="G15" s="30">
         <v>95039</v>
       </c>
-      <c r="H28" s="41">
+      <c r="H15" s="31">
         <v>342248</v>
       </c>
-      <c r="I28" s="37">
+      <c r="I15" s="27">
         <v>272881</v>
       </c>
-      <c r="J28" s="38">
+      <c r="J15" s="28">
         <v>69367</v>
       </c>
     </row>
-    <row r="29" spans="1:233" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="36" t="s">
-        <v>19</v>
+    <row r="16" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="26" t="s">
+        <v>20</v>
       </c>
-      <c r="B29" s="37">
+      <c r="B16" s="27">
         <v>-78639</v>
       </c>
-      <c r="C29" s="37">
+      <c r="C16" s="27">
         <v>-104350</v>
       </c>
-      <c r="D29" s="38">
+      <c r="D16" s="28">
         <v>25711</v>
       </c>
-      <c r="E29" s="39">
+      <c r="E16" s="29">
         <v>271115</v>
       </c>
-      <c r="F29" s="37">
+      <c r="F16" s="27">
         <v>174671</v>
       </c>
-      <c r="G29" s="40">
+      <c r="G16" s="30">
         <v>96444</v>
       </c>
-      <c r="H29" s="41">
+      <c r="H16" s="31">
         <v>349754</v>
       </c>
-      <c r="I29" s="37">
+      <c r="I16" s="27">
         <v>279021</v>
       </c>
-      <c r="J29" s="38">
+      <c r="J16" s="28">
         <v>70733</v>
       </c>
     </row>
-    <row r="30" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="36" t="s">
-        <v>20</v>
+    <row r="17" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="26" t="s">
+        <v>21</v>
       </c>
-      <c r="B30" s="37">
+      <c r="B17" s="27">
         <v>-71214</v>
       </c>
-      <c r="C30" s="37">
+      <c r="C17" s="27">
         <v>-97117</v>
       </c>
-      <c r="D30" s="38">
+      <c r="D17" s="28">
         <v>25904</v>
       </c>
-      <c r="E30" s="39">
+      <c r="E17" s="29">
         <v>275719</v>
       </c>
-      <c r="F30" s="37">
+      <c r="F17" s="27">
         <v>177954</v>
       </c>
-      <c r="G30" s="40">
+      <c r="G17" s="30">
         <v>97765</v>
       </c>
-      <c r="H30" s="41">
+      <c r="H17" s="31">
         <v>346933</v>
       </c>
-      <c r="I30" s="37">
+      <c r="I17" s="27">
         <v>275071</v>
       </c>
-      <c r="J30" s="38">
+      <c r="J17" s="28">
         <v>71862</v>
       </c>
     </row>
-    <row r="31" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="36" t="s">
-        <v>21</v>
+    <row r="18" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="26" t="s">
+        <v>22</v>
       </c>
-      <c r="B31" s="37">
+      <c r="B18" s="27">
         <v>-81498</v>
       </c>
-      <c r="C31" s="37">
+      <c r="C18" s="27">
         <v>-107722</v>
       </c>
-      <c r="D31" s="38">
+      <c r="D18" s="28">
         <v>26224</v>
       </c>
-      <c r="E31" s="39">
+      <c r="E18" s="29">
         <v>273687</v>
       </c>
-      <c r="F31" s="37">
+      <c r="F18" s="27">
         <v>175484</v>
       </c>
-      <c r="G31" s="40">
+      <c r="G18" s="30">
         <v>98203</v>
       </c>
-      <c r="H31" s="41">
+      <c r="H18" s="31">
         <v>355185</v>
       </c>
-      <c r="I31" s="37">
+      <c r="I18" s="27">
         <v>283206</v>
       </c>
-      <c r="J31" s="38">
+      <c r="J18" s="28">
         <v>71979</v>
       </c>
     </row>
-    <row r="32" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="36" t="s">
-        <v>22</v>
+    <row r="19" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="26" t="s">
+        <v>23</v>
       </c>
-      <c r="B32" s="37">
+      <c r="B19" s="27">
         <v>-74250</v>
       </c>
-      <c r="C32" s="37">
+      <c r="C19" s="27">
         <v>-100088</v>
       </c>
-      <c r="D32" s="38">
+      <c r="D19" s="28">
         <v>25839</v>
       </c>
-      <c r="E32" s="39">
+      <c r="E19" s="29">
         <v>269501</v>
       </c>
-      <c r="F32" s="37">
+      <c r="F19" s="27">
         <v>170941</v>
       </c>
-      <c r="G32" s="40">
+      <c r="G19" s="30">
         <v>98560</v>
       </c>
-      <c r="H32" s="41">
+      <c r="H19" s="31">
         <v>343751</v>
       </c>
-      <c r="I32" s="37">
+      <c r="I19" s="27">
         <v>271029</v>
       </c>
-      <c r="J32" s="38">
+      <c r="J19" s="28">
         <v>72722</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="36" t="s">
-        <v>23</v>
+    <row r="20" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="26" t="s">
+        <v>24</v>
       </c>
-      <c r="B33" s="37">
+      <c r="B20" s="27">
         <v>-79752</v>
       </c>
-      <c r="C33" s="37">
+      <c r="C20" s="27">
         <v>-106002</v>
       </c>
-      <c r="D33" s="38">
+      <c r="D20" s="28">
         <v>26249</v>
       </c>
-      <c r="E33" s="39">
+      <c r="E20" s="29">
         <v>275828</v>
       </c>
-      <c r="F33" s="37">
+      <c r="F20" s="27">
         <v>176509</v>
       </c>
-      <c r="G33" s="40">
+      <c r="G20" s="30">
         <v>99319</v>
       </c>
-      <c r="H33" s="41">
+      <c r="H20" s="31">
         <v>355580</v>
       </c>
-      <c r="I33" s="37">
+      <c r="I20" s="27">
         <v>282510</v>
       </c>
-      <c r="J33" s="38">
+      <c r="J20" s="28">
         <v>73070</v>
       </c>
+      <c r="K20" s="38"/>
+      <c r="L20" s="38"/>
+      <c r="M20" s="38"/>
+      <c r="N20" s="38"/>
+      <c r="O20" s="38"/>
+      <c r="P20" s="38"/>
+      <c r="Q20" s="38"/>
+      <c r="R20" s="38"/>
+      <c r="S20" s="38"/>
+      <c r="T20" s="38"/>
+      <c r="U20" s="38"/>
+      <c r="V20" s="38"/>
+      <c r="W20" s="38"/>
+      <c r="X20" s="38"/>
+      <c r="Y20" s="38"/>
+      <c r="Z20" s="38"/>
+      <c r="AA20" s="38"/>
+      <c r="AB20" s="38"/>
+      <c r="AC20" s="38"/>
+      <c r="AD20" s="38"/>
+      <c r="AE20" s="38"/>
+      <c r="AF20" s="38"/>
+      <c r="AG20" s="38"/>
+      <c r="AH20" s="38"/>
+      <c r="AI20" s="38"/>
+      <c r="AJ20" s="38"/>
+      <c r="AK20" s="38"/>
+      <c r="AL20" s="38"/>
+      <c r="AM20" s="38"/>
+      <c r="AN20" s="38"/>
+      <c r="AO20" s="38"/>
+      <c r="AP20" s="38"/>
+      <c r="AQ20" s="38"/>
+      <c r="AR20" s="38"/>
+      <c r="AS20" s="38"/>
+      <c r="AT20" s="38"/>
+      <c r="AU20" s="38"/>
+      <c r="AV20" s="38"/>
+      <c r="AW20" s="38"/>
+      <c r="AX20" s="38"/>
+      <c r="AY20" s="38"/>
+      <c r="AZ20" s="38"/>
+      <c r="BA20" s="38"/>
+      <c r="BB20" s="38"/>
+      <c r="BC20" s="38"/>
+      <c r="BD20" s="38"/>
+      <c r="BE20" s="38"/>
+      <c r="BF20" s="38"/>
+      <c r="BG20" s="38"/>
+      <c r="BH20" s="38"/>
+      <c r="BI20" s="38"/>
+      <c r="BJ20" s="38"/>
+      <c r="BK20" s="38"/>
+      <c r="BL20" s="38"/>
+      <c r="BM20" s="38"/>
+      <c r="BN20" s="38"/>
+      <c r="BO20" s="38"/>
+      <c r="BP20" s="38"/>
+      <c r="BQ20" s="38"/>
+      <c r="BR20" s="38"/>
+      <c r="BS20" s="38"/>
+      <c r="BT20" s="38"/>
+      <c r="BU20" s="38"/>
+      <c r="BV20" s="38"/>
+      <c r="BW20" s="38"/>
+      <c r="BX20" s="38"/>
+      <c r="BY20" s="38"/>
+      <c r="BZ20" s="38"/>
+      <c r="CA20" s="38"/>
+      <c r="CB20" s="38"/>
+      <c r="CC20" s="38"/>
+      <c r="CD20" s="38"/>
+      <c r="CE20" s="38"/>
+      <c r="CF20" s="38"/>
+      <c r="CG20" s="38"/>
+      <c r="CH20" s="38"/>
+      <c r="CI20" s="38"/>
+      <c r="CJ20" s="38"/>
+      <c r="CK20" s="38"/>
+      <c r="CL20" s="38"/>
+      <c r="CM20" s="38"/>
+      <c r="CN20" s="38"/>
+      <c r="CO20" s="38"/>
+      <c r="CP20" s="38"/>
+      <c r="CQ20" s="38"/>
+      <c r="CR20" s="38"/>
+      <c r="CS20" s="38"/>
+      <c r="CT20" s="38"/>
+      <c r="CU20" s="38"/>
+      <c r="CV20" s="38"/>
+      <c r="CW20" s="38"/>
+      <c r="CX20" s="38"/>
+      <c r="CY20" s="38"/>
+      <c r="CZ20" s="38"/>
+      <c r="DA20" s="38"/>
+      <c r="DB20" s="38"/>
+      <c r="DC20" s="38"/>
+      <c r="DD20" s="38"/>
+      <c r="DE20" s="38"/>
+      <c r="DF20" s="38"/>
+      <c r="DG20" s="38"/>
+      <c r="DH20" s="38"/>
+      <c r="DI20" s="38"/>
+      <c r="DJ20" s="38"/>
+      <c r="DK20" s="38"/>
+      <c r="DL20" s="38"/>
+      <c r="DM20" s="38"/>
+      <c r="DN20" s="38"/>
+      <c r="DO20" s="38"/>
+      <c r="DP20" s="38"/>
+      <c r="DQ20" s="38"/>
+      <c r="DR20" s="38"/>
+      <c r="DS20" s="38"/>
+      <c r="DT20" s="38"/>
+      <c r="DU20" s="38"/>
+      <c r="DV20" s="38"/>
+      <c r="DW20" s="38"/>
+      <c r="DX20" s="38"/>
+      <c r="DY20" s="38"/>
+      <c r="DZ20" s="38"/>
+      <c r="EA20" s="38"/>
+      <c r="EB20" s="38"/>
+      <c r="EC20" s="38"/>
+      <c r="ED20" s="38"/>
+      <c r="EE20" s="38"/>
+      <c r="EF20" s="38"/>
+      <c r="EG20" s="38"/>
+      <c r="EH20" s="38"/>
+      <c r="EI20" s="38"/>
+      <c r="EJ20" s="38"/>
+      <c r="EK20" s="38"/>
+      <c r="EL20" s="38"/>
+      <c r="EM20" s="38"/>
+      <c r="EN20" s="38"/>
+      <c r="EO20" s="38"/>
+      <c r="EP20" s="38"/>
+      <c r="EQ20" s="38"/>
+      <c r="ER20" s="38"/>
+      <c r="ES20" s="38"/>
+      <c r="ET20" s="38"/>
+      <c r="EU20" s="38"/>
+      <c r="EV20" s="38"/>
+      <c r="EW20" s="38"/>
+      <c r="EX20" s="38"/>
+      <c r="EY20" s="38"/>
+      <c r="EZ20" s="38"/>
+      <c r="FA20" s="38"/>
+      <c r="FB20" s="38"/>
+      <c r="FC20" s="38"/>
+      <c r="FD20" s="38"/>
+      <c r="FE20" s="38"/>
+      <c r="FF20" s="38"/>
+      <c r="FG20" s="38"/>
+      <c r="FH20" s="38"/>
+      <c r="FI20" s="38"/>
+      <c r="FJ20" s="38"/>
+      <c r="FK20" s="38"/>
+      <c r="FL20" s="38"/>
+      <c r="FM20" s="38"/>
+      <c r="FN20" s="38"/>
+      <c r="FO20" s="38"/>
+      <c r="FP20" s="38"/>
+      <c r="FQ20" s="38"/>
+      <c r="FR20" s="38"/>
+      <c r="FS20" s="38"/>
+      <c r="FT20" s="38"/>
+      <c r="FU20" s="38"/>
+      <c r="FV20" s="38"/>
+      <c r="FW20" s="38"/>
+      <c r="FX20" s="38"/>
+      <c r="FY20" s="38"/>
+      <c r="FZ20" s="38"/>
+      <c r="GA20" s="38"/>
+      <c r="GB20" s="38"/>
+      <c r="GC20" s="38"/>
+      <c r="GD20" s="38"/>
+      <c r="GE20" s="38"/>
+      <c r="GF20" s="38"/>
+      <c r="GG20" s="38"/>
+      <c r="GH20" s="38"/>
+      <c r="GI20" s="38"/>
+      <c r="GJ20" s="38"/>
+      <c r="GK20" s="38"/>
+      <c r="GL20" s="38"/>
+      <c r="GM20" s="38"/>
+      <c r="GN20" s="38"/>
+      <c r="GO20" s="38"/>
+      <c r="GP20" s="38"/>
+      <c r="GQ20" s="38"/>
+      <c r="GR20" s="38"/>
+      <c r="GS20" s="38"/>
+      <c r="GT20" s="38"/>
+      <c r="GU20" s="38"/>
+      <c r="GV20" s="38"/>
+      <c r="GW20" s="38"/>
+      <c r="GX20" s="38"/>
+      <c r="GY20" s="38"/>
+      <c r="GZ20" s="38"/>
+      <c r="HA20" s="38"/>
+      <c r="HB20" s="38"/>
+      <c r="HC20" s="38"/>
+      <c r="HD20" s="38"/>
+      <c r="HE20" s="38"/>
+      <c r="HF20" s="38"/>
+      <c r="HG20" s="38"/>
+      <c r="HH20" s="38"/>
+      <c r="HI20" s="38"/>
+      <c r="HJ20" s="38"/>
+      <c r="HK20" s="38"/>
+      <c r="HL20" s="38"/>
+      <c r="HM20" s="38"/>
+      <c r="HN20" s="38"/>
+      <c r="HO20" s="38"/>
+      <c r="HP20" s="38"/>
+      <c r="HQ20" s="38"/>
+      <c r="HR20" s="38"/>
+      <c r="HS20" s="38"/>
+      <c r="HT20" s="38"/>
+      <c r="HU20" s="38"/>
+      <c r="HV20" s="38"/>
+      <c r="HW20" s="38"/>
+      <c r="HX20" s="38"/>
+      <c r="HY20" s="38"/>
     </row>
-    <row r="34" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="36" t="s">
-        <v>24</v>
+    <row r="21" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="26" t="s">
+        <v>25</v>
       </c>
-      <c r="B34" s="37">
+      <c r="B21" s="27">
         <v>-96948</v>
       </c>
-      <c r="C34" s="37">
+      <c r="C21" s="27">
         <v>-122822</v>
       </c>
-      <c r="D34" s="38">
+      <c r="D21" s="28">
         <v>25874</v>
       </c>
-      <c r="E34" s="39">
+      <c r="E21" s="29">
         <v>270192</v>
       </c>
-      <c r="F34" s="37">
+      <c r="F21" s="27">
         <v>170476</v>
       </c>
-      <c r="G34" s="40">
+      <c r="G21" s="30">
         <v>99715</v>
       </c>
-      <c r="H34" s="41">
+      <c r="H21" s="31">
         <v>367140</v>
       </c>
-      <c r="I34" s="37">
+      <c r="I21" s="27">
         <v>293299</v>
       </c>
-      <c r="J34" s="38">
+      <c r="J21" s="28">
         <v>73841</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="43" t="s">
+    <row r="22" spans="1:233" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="B35" s="44"/>
-      <c r="C35" s="44"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="46"/>
-      <c r="F35" s="44"/>
-      <c r="G35" s="47"/>
-      <c r="H35" s="48"/>
-      <c r="I35" s="44"/>
-      <c r="J35" s="45"/>
+      <c r="B22" s="40"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="44"/>
+      <c r="I22" s="40"/>
+      <c r="J22" s="41"/>
     </row>
-    <row r="36" spans="1:10" ht="25.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="30" t="s">
-        <v>12</v>
+    <row r="23" spans="1:233" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="26" t="s">
+        <v>27</v>
       </c>
-      <c r="B36" s="31">
-        <v>-901469</v>
+      <c r="B23" s="27">
+        <v>-911689</v>
       </c>
-      <c r="C36" s="31">
-        <v>-1240941</v>
+      <c r="C23" s="27">
+        <v>-1240816</v>
       </c>
-      <c r="D36" s="32">
-        <v>339472</v>
+      <c r="D23" s="28">
+        <v>329127</v>
       </c>
-      <c r="E36" s="33">
-        <v>3432339</v>
+      <c r="E23" s="29">
+        <v>3429920</v>
       </c>
-      <c r="F36" s="31">
-        <v>2197486</v>
+      <c r="F23" s="27">
+        <v>2197515</v>
       </c>
-      <c r="G36" s="34">
-        <v>1234853</v>
+      <c r="G23" s="30">
+        <v>1232405</v>
       </c>
-      <c r="H36" s="35">
-        <v>4333808</v>
+      <c r="H23" s="31">
+        <v>4341609</v>
       </c>
-      <c r="I36" s="31">
-        <v>3438427</v>
+      <c r="I23" s="27">
+        <v>3438331</v>
       </c>
-      <c r="J36" s="32">
-        <v>895381</v>
+      <c r="J23" s="28">
+        <v>903278</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="36" t="s">
-        <v>27</v>
+    <row r="24" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="32" t="s">
+        <v>28</v>
       </c>
-      <c r="B37" s="37">
-        <v>-128344</v>
+      <c r="B24" s="33">
+        <v>-128331</v>
       </c>
-      <c r="C37" s="37">
+      <c r="C24" s="33">
         <v>-155620</v>
       </c>
-      <c r="D37" s="38">
-        <v>27276</v>
+      <c r="D24" s="34">
+        <v>27290</v>
       </c>
-      <c r="E37" s="39">
-        <v>273621</v>
+      <c r="E24" s="35">
+        <v>273740</v>
       </c>
-      <c r="F37" s="37">
+      <c r="F24" s="33">
         <v>173411</v>
       </c>
-      <c r="G37" s="40">
-        <v>100210</v>
+      <c r="G24" s="36">
+        <v>100329</v>
       </c>
-      <c r="H37" s="41">
-        <v>401965</v>
+      <c r="H24" s="37">
+        <v>402070</v>
       </c>
-      <c r="I37" s="37">
+      <c r="I24" s="33">
         <v>329031</v>
       </c>
-      <c r="J37" s="38">
-        <v>72934</v>
+      <c r="J24" s="34">
+        <v>73039</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="36" t="s">
-        <v>28</v>
+    <row r="25" spans="1:233" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="26" t="s">
+        <v>29</v>
       </c>
-      <c r="B38" s="37">
-        <v>-119822</v>
+      <c r="B25" s="27">
+        <v>-128331</v>
       </c>
-      <c r="C38" s="37">
-        <v>-146734</v>
+      <c r="C25" s="27">
+        <v>-155620</v>
       </c>
-      <c r="D38" s="38">
-        <v>26912</v>
+      <c r="D25" s="28">
+        <v>27290</v>
       </c>
-      <c r="E38" s="39">
-        <v>280583</v>
+      <c r="E25" s="29">
+        <v>273740</v>
       </c>
-      <c r="F38" s="37">
+      <c r="F25" s="27">
+        <v>173411</v>
+      </c>
+      <c r="G25" s="30">
+        <v>100329</v>
+      </c>
+      <c r="H25" s="31">
+        <v>402070</v>
+      </c>
+      <c r="I25" s="27">
+        <v>329031</v>
+      </c>
+      <c r="J25" s="28">
+        <v>73039</v>
+      </c>
+    </row>
+    <row r="26" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="27">
+        <v>-119780</v>
+      </c>
+      <c r="C26" s="27">
+        <v>-146733</v>
+      </c>
+      <c r="D26" s="28">
+        <v>26954</v>
+      </c>
+      <c r="E26" s="29">
+        <v>280663</v>
+      </c>
+      <c r="F26" s="27">
         <v>180643</v>
       </c>
-      <c r="G38" s="40">
-        <v>99940</v>
+      <c r="G26" s="30">
+        <v>100020</v>
       </c>
-      <c r="H38" s="41">
-        <v>400405</v>
+      <c r="H26" s="31">
+        <v>400443</v>
       </c>
-      <c r="I38" s="37">
+      <c r="I26" s="27">
         <v>327377</v>
       </c>
-      <c r="J38" s="38">
-        <v>73029</v>
+      <c r="J26" s="28">
+        <v>73066</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="36" t="s">
-        <v>29</v>
+    <row r="27" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="26" t="s">
+        <v>31</v>
       </c>
-      <c r="B39" s="37">
-        <v>-135963</v>
+      <c r="B27" s="27">
+        <v>-135856</v>
       </c>
-      <c r="C39" s="37">
+      <c r="C27" s="27">
         <v>-162060</v>
       </c>
-      <c r="D39" s="38">
-        <v>26097</v>
+      <c r="D27" s="28">
+        <v>26204</v>
       </c>
-      <c r="E39" s="39">
-        <v>283269</v>
+      <c r="E27" s="29">
+        <v>283132</v>
       </c>
-      <c r="F39" s="37">
+      <c r="F27" s="27">
         <v>183902</v>
       </c>
-      <c r="G39" s="40">
-        <v>99367</v>
+      <c r="G27" s="30">
+        <v>99230</v>
       </c>
-      <c r="H39" s="41">
-        <v>419232</v>
+      <c r="H27" s="31">
+        <v>418988</v>
       </c>
-      <c r="I39" s="37">
+      <c r="I27" s="27">
         <v>345962</v>
       </c>
-      <c r="J39" s="38">
-        <v>73270</v>
+      <c r="J27" s="28">
+        <v>73026</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="41" t="s">
-        <v>30</v>
+    <row r="28" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="26" t="s">
+        <v>32</v>
       </c>
-      <c r="B40" s="37">
-        <v>-60117</v>
+      <c r="B28" s="27">
+        <v>-60084</v>
       </c>
-      <c r="C40" s="37">
+      <c r="C28" s="27">
         <v>-86522</v>
       </c>
-      <c r="D40" s="38">
-        <v>26405</v>
+      <c r="D28" s="28">
+        <v>26439</v>
       </c>
-      <c r="E40" s="39">
-        <v>291184</v>
+      <c r="E28" s="29">
+        <v>291033</v>
       </c>
-      <c r="F40" s="37">
+      <c r="F28" s="27">
         <v>190502</v>
       </c>
-      <c r="G40" s="40">
-        <v>100682</v>
+      <c r="G28" s="30">
+        <v>100530</v>
       </c>
-      <c r="H40" s="41">
-        <v>351302</v>
+      <c r="H28" s="31">
+        <v>351116</v>
       </c>
-      <c r="I40" s="37">
+      <c r="I28" s="27">
         <v>277025</v>
       </c>
-      <c r="J40" s="38">
-        <v>74277</v>
+      <c r="J28" s="28">
+        <v>74092</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="41" t="s">
-        <v>31</v>
+    <row r="29" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="26" t="s">
+        <v>33</v>
       </c>
-      <c r="B41" s="37">
-        <v>-70595</v>
+      <c r="B29" s="27">
+        <v>-70564</v>
       </c>
-      <c r="C41" s="37">
+      <c r="C29" s="27">
         <v>-96955</v>
       </c>
-      <c r="D41" s="38">
-        <v>26359</v>
+      <c r="D29" s="28">
+        <v>26391</v>
       </c>
-      <c r="E41" s="39">
-        <v>280081</v>
+      <c r="E29" s="29">
+        <v>280056</v>
       </c>
-      <c r="F41" s="37">
+      <c r="F29" s="27">
         <v>179710</v>
       </c>
-      <c r="G41" s="40">
-        <v>100371</v>
+      <c r="G29" s="30">
+        <v>100346</v>
       </c>
-      <c r="H41" s="41">
-        <v>350676</v>
+      <c r="H29" s="31">
+        <v>350620</v>
       </c>
-      <c r="I41" s="37">
+      <c r="I29" s="27">
         <v>276664</v>
       </c>
-      <c r="J41" s="38">
-        <v>74011</v>
+      <c r="J29" s="28">
+        <v>73955</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="41" t="s">
-        <v>32</v>
+    <row r="30" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="26" t="s">
+        <v>34</v>
       </c>
-      <c r="B42" s="37">
-        <v>-57728</v>
+      <c r="B30" s="27">
+        <v>-57637</v>
       </c>
-      <c r="C42" s="37">
+      <c r="C30" s="27">
         <v>-85567</v>
       </c>
-      <c r="D42" s="38">
-        <v>27839</v>
+      <c r="D30" s="28">
+        <v>27930</v>
       </c>
-      <c r="E42" s="39">
-        <v>280195</v>
+      <c r="E30" s="29">
+        <v>280442</v>
       </c>
-      <c r="F42" s="37">
+      <c r="F30" s="27">
         <v>178756</v>
       </c>
-      <c r="G42" s="40">
-        <v>101439</v>
+      <c r="G30" s="30">
+        <v>101685</v>
       </c>
-      <c r="H42" s="41">
-        <v>337923</v>
+      <c r="H30" s="31">
+        <v>338078</v>
       </c>
-      <c r="I42" s="37">
+      <c r="I30" s="27">
         <v>264323</v>
       </c>
-      <c r="J42" s="38">
-        <v>73600</v>
+      <c r="J30" s="28">
+        <v>73755</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="41" t="s">
-        <v>33</v>
+    <row r="31" spans="1:233" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="26" t="s">
+        <v>35</v>
       </c>
-      <c r="B43" s="37">
-        <v>-73942</v>
+      <c r="B31" s="27">
+        <v>-74233</v>
       </c>
-      <c r="C43" s="37">
-        <v>-102548</v>
+      <c r="C31" s="27">
+        <v>-102547</v>
       </c>
-      <c r="D43" s="38">
-        <v>28606</v>
+      <c r="D31" s="28">
+        <v>28315</v>
       </c>
-      <c r="E43" s="39">
-        <v>283598</v>
+      <c r="E31" s="29">
+        <v>284322</v>
       </c>
-      <c r="F43" s="37">
-        <v>180101</v>
+      <c r="F31" s="27">
+        <v>180102</v>
       </c>
-      <c r="G43" s="40">
-        <v>103497</v>
+      <c r="G31" s="30">
+        <v>104220</v>
       </c>
-      <c r="H43" s="41">
-        <v>357540</v>
+      <c r="H31" s="31">
+        <v>358555</v>
       </c>
-      <c r="I43" s="37">
-        <v>282650</v>
+      <c r="I31" s="27">
+        <v>282649</v>
       </c>
-      <c r="J43" s="38">
-        <v>74891</v>
+      <c r="J31" s="28">
+        <v>75906</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="41" t="s">
-        <v>34</v>
+    <row r="32" spans="1:233" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="26" t="s">
+        <v>36</v>
       </c>
-      <c r="B44" s="37">
-        <v>-55173</v>
+      <c r="B32" s="27">
+        <v>-56011</v>
       </c>
-      <c r="C44" s="37">
-        <v>-85589</v>
+      <c r="C32" s="27">
+        <v>-85594</v>
       </c>
-      <c r="D44" s="38">
-        <v>30416</v>
+      <c r="D32" s="28">
+        <v>29583</v>
       </c>
-      <c r="E44" s="39">
-        <v>283736</v>
+      <c r="E32" s="29">
+        <v>284344</v>
       </c>
-      <c r="F44" s="37">
-        <v>178452</v>
+      <c r="F32" s="27">
+        <v>178446</v>
       </c>
-      <c r="G44" s="40">
-        <v>105284</v>
+      <c r="G32" s="30">
+        <v>105898</v>
       </c>
-      <c r="H44" s="41">
-        <v>338909</v>
+      <c r="H32" s="31">
+        <v>340355</v>
       </c>
-      <c r="I44" s="37">
-        <v>264041</v>
+      <c r="I32" s="27">
+        <v>264040</v>
       </c>
-      <c r="J44" s="38">
-        <v>74868</v>
+      <c r="J32" s="28">
+        <v>76315</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="41" t="s">
-        <v>35</v>
+    <row r="33" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="26" t="s">
+        <v>37</v>
       </c>
-      <c r="B45" s="37">
-        <v>-47681</v>
+      <c r="B33" s="27">
+        <v>-49168</v>
       </c>
-      <c r="C45" s="37">
-        <v>-77850</v>
+      <c r="C33" s="27">
+        <v>-77760</v>
       </c>
-      <c r="D45" s="38">
-        <v>30169</v>
+      <c r="D33" s="28">
+        <v>28592</v>
       </c>
-      <c r="E45" s="39">
-        <v>293901</v>
+      <c r="E33" s="29">
+        <v>293804</v>
       </c>
-      <c r="F45" s="37">
-        <v>188470</v>
+      <c r="F33" s="27">
+        <v>188478</v>
       </c>
-      <c r="G45" s="40">
-        <v>105431</v>
+      <c r="G33" s="30">
+        <v>105327</v>
       </c>
-      <c r="H45" s="41">
-        <v>341582</v>
+      <c r="H33" s="31">
+        <v>342972</v>
       </c>
-      <c r="I45" s="37">
-        <v>266320</v>
+      <c r="I33" s="27">
+        <v>266237</v>
       </c>
-      <c r="J45" s="38">
-        <v>75262</v>
+      <c r="J33" s="28">
+        <v>76735</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="36" t="s">
-        <v>36</v>
+    <row r="34" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="26" t="s">
+        <v>38</v>
       </c>
-      <c r="B46" s="37">
-        <v>-28749</v>
+      <c r="B34" s="27">
+        <v>-31102</v>
       </c>
-      <c r="C46" s="37">
-        <v>-58526</v>
+      <c r="C34" s="27">
+        <v>-58577</v>
       </c>
-      <c r="D46" s="38">
-        <v>29777</v>
+      <c r="D34" s="28">
+        <v>27476</v>
       </c>
-      <c r="E46" s="39">
-        <v>302594</v>
+      <c r="E34" s="29">
+        <v>301177</v>
       </c>
-      <c r="F46" s="37">
-        <v>196420</v>
+      <c r="F34" s="27">
+        <v>196427</v>
       </c>
-      <c r="G46" s="40">
-        <v>106174</v>
+      <c r="G34" s="30">
+        <v>104750</v>
       </c>
-      <c r="H46" s="41">
-        <v>331343</v>
+      <c r="H34" s="31">
+        <v>332279</v>
       </c>
-      <c r="I46" s="37">
-        <v>254946</v>
+      <c r="I34" s="27">
+        <v>255004</v>
       </c>
-      <c r="J46" s="38">
-        <v>76397</v>
+      <c r="J34" s="28">
+        <v>77275</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="36" t="s">
-        <v>37</v>
+    <row r="35" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="26" t="s">
+        <v>39</v>
       </c>
-      <c r="B47" s="37">
-        <v>-53044</v>
+      <c r="B35" s="27">
+        <v>-56026</v>
       </c>
-      <c r="C47" s="37">
-        <v>-83641</v>
+      <c r="C35" s="27">
+        <v>-83634</v>
       </c>
-      <c r="D47" s="38">
-        <v>30597</v>
+      <c r="D35" s="28">
+        <v>27608</v>
       </c>
-      <c r="E47" s="39">
-        <v>292290</v>
+      <c r="E35" s="29">
+        <v>290906</v>
       </c>
-      <c r="F47" s="37">
-        <v>186287</v>
+      <c r="F35" s="27">
+        <v>186274</v>
       </c>
-      <c r="G47" s="40">
-        <v>106002</v>
+      <c r="G35" s="30">
+        <v>104632</v>
       </c>
-      <c r="H47" s="41">
-        <v>345334</v>
+      <c r="H35" s="31">
+        <v>346932</v>
       </c>
-      <c r="I47" s="37">
-        <v>269928</v>
+      <c r="I35" s="27">
+        <v>269908</v>
       </c>
-      <c r="J47" s="38">
-        <v>75406</v>
+      <c r="J35" s="28">
+        <v>77024</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="30" t="s">
+    <row r="36" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="B36" s="27">
+        <v>-72900</v>
+      </c>
+      <c r="C36" s="27">
+        <v>-99246</v>
+      </c>
+      <c r="D36" s="28">
+        <v>26347</v>
+      </c>
+      <c r="E36" s="29">
+        <v>286301</v>
+      </c>
+      <c r="F36" s="27">
+        <v>180864</v>
+      </c>
+      <c r="G36" s="30">
+        <v>105437</v>
+      </c>
+      <c r="H36" s="31">
+        <v>359201</v>
+      </c>
+      <c r="I36" s="27">
+        <v>280110</v>
+      </c>
+      <c r="J36" s="28">
+        <v>79090</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="39" t="s">
+        <v>41</v>
+      </c>
+      <c r="B37" s="40"/>
+      <c r="C37" s="40"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="42"/>
+      <c r="F37" s="40"/>
+      <c r="G37" s="43"/>
+      <c r="H37" s="44"/>
+      <c r="I37" s="40"/>
+      <c r="J37" s="41"/>
+    </row>
+    <row r="38" spans="1:10" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="B38" s="33">
+        <v>-54455</v>
+      </c>
+      <c r="C38" s="33">
+        <v>-81791</v>
+      </c>
+      <c r="D38" s="34">
+        <v>27336</v>
+      </c>
+      <c r="E38" s="35">
+        <v>302149</v>
+      </c>
+      <c r="F38" s="33">
+        <v>195492</v>
+      </c>
+      <c r="G38" s="36">
+        <v>106658</v>
+      </c>
+      <c r="H38" s="37">
+        <v>356604</v>
+      </c>
+      <c r="I38" s="33">
+        <v>277283</v>
+      </c>
+      <c r="J38" s="34">
+        <v>79321</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B39" s="27">
+        <v>-54455</v>
+      </c>
+      <c r="C39" s="27">
+        <v>-81791</v>
+      </c>
+      <c r="D39" s="28">
+        <v>27336</v>
+      </c>
+      <c r="E39" s="29">
+        <v>302149</v>
+      </c>
+      <c r="F39" s="27">
+        <v>195492</v>
+      </c>
+      <c r="G39" s="30">
+        <v>106658</v>
+      </c>
+      <c r="H39" s="31">
+        <v>356604</v>
+      </c>
+      <c r="I39" s="27">
+        <v>277283</v>
+      </c>
+      <c r="J39" s="28">
+        <v>79321</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="B40" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C40" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D40" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E40" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="F40" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="G40" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="H40" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="I40" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="J40" s="28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="B41" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C41" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D41" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E41" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="F41" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="G41" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="H41" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="I41" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="J41" s="28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C42" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D42" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E42" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="F42" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="G42" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="H42" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="I42" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="J42" s="28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="B43" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C43" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D43" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E43" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="F43" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="G43" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="H43" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="I43" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="J43" s="28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="B44" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C44" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D44" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E44" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="F44" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="G44" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="H44" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="I44" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="J44" s="28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="B45" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C45" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D45" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E45" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="F45" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="G45" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="H45" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="I45" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="J45" s="28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="B46" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C46" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D46" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E46" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="F46" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="G46" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="H46" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="I46" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="J46" s="28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="B47" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C47" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D47" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E47" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="F47" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="G47" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="H47" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="I47" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="J47" s="28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B48" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C48" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D48" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E48" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="F48" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="G48" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="H48" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="I48" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="J48" s="28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="B48" s="31">
+      <c r="B49" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C49" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D49" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E49" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="F49" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="G49" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="H49" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="I49" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="J49" s="28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B50" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C50" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D50" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E50" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="F50" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="G50" s="36" t="s">
+        <v>42</v>
+      </c>
+      <c r="H50" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="I50" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="J50" s="28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="45" t="s">
+        <v>43</v>
+      </c>
+      <c r="B51" s="46"/>
+      <c r="C51" s="46"/>
+      <c r="D51" s="46"/>
+      <c r="E51" s="46"/>
+      <c r="F51" s="46"/>
+      <c r="G51" s="46"/>
+      <c r="H51" s="46"/>
+      <c r="I51" s="47"/>
+      <c r="J51" s="47"/>
+    </row>
+    <row r="52" spans="1:10" s="50" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="48"/>
+      <c r="B52" s="49">
         <v>-70311</v>
       </c>
-      <c r="C48" s="31">
+      <c r="C52" s="49">
         <v>-99329</v>
       </c>
-      <c r="D48" s="32">
+      <c r="D52" s="49">
         <v>29018</v>
       </c>
-      <c r="E48" s="33">
+      <c r="E52" s="49">
         <v>287287</v>
       </c>
-      <c r="F48" s="31">
+      <c r="F52" s="49">
         <v>180832</v>
       </c>
-      <c r="G48" s="34">
+      <c r="G52" s="49">
         <v>106455</v>
       </c>
-      <c r="H48" s="35">
+      <c r="H52" s="49">
         <v>357598</v>
       </c>
-      <c r="I48" s="31">
+      <c r="I52" s="49">
         <v>280161</v>
       </c>
-      <c r="J48" s="32">
+      <c r="J52" s="49">
         <v>77437</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="49" t="s">
-        <v>38</v>
+    <row r="53" spans="1:10" s="50" customFormat="1" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="48" t="s">
+        <v>44</v>
       </c>
-      <c r="B49" s="50"/>
-      <c r="C49" s="50"/>
-      <c r="D49" s="50"/>
-      <c r="E49" s="50"/>
-      <c r="F49" s="50"/>
-      <c r="G49" s="50"/>
-      <c r="H49" s="50"/>
-      <c r="I49" s="51"/>
-      <c r="J49" s="51"/>
+      <c r="B53" s="11"/>
+      <c r="C53" s="11"/>
+      <c r="D53" s="11"/>
+      <c r="E53" s="11"/>
+      <c r="F53" s="11"/>
+      <c r="G53" s="11"/>
+      <c r="H53" s="11"/>
+      <c r="I53" s="48"/>
+      <c r="J53" s="48"/>
     </row>
-    <row r="50" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="52"/>
-      <c r="B50" s="51">
-        <v>-56825</v>
+    <row r="54" spans="1:10" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="48" t="s">
+        <v>45</v>
       </c>
-      <c r="C50" s="51">
-        <v>-86900</v>
-      </c>
-      <c r="D50" s="51">
-        <v>30075</v>
-      </c>
-      <c r="E50" s="51">
-        <v>292052</v>
-      </c>
-      <c r="F50" s="51">
-        <v>185641</v>
-      </c>
-      <c r="G50" s="51">
-        <v>106411</v>
-      </c>
-      <c r="H50" s="51">
-        <v>348877</v>
-      </c>
-      <c r="I50" s="51">
-        <v>272541</v>
-      </c>
-      <c r="J50" s="51">
-        <v>76336</v>
+      <c r="B54" s="48"/>
+      <c r="C54" s="48"/>
+      <c r="D54" s="48"/>
+      <c r="E54" s="48"/>
+      <c r="F54" s="48"/>
+      <c r="G54" s="48"/>
+      <c r="H54" s="48"/>
+      <c r="I54" s="48"/>
+      <c r="J54" s="48"/>
+    </row>
+    <row r="55" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>46</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="49" t="s">
-        <v>39</v>
-      </c>
-      <c r="B51" s="11"/>
-      <c r="C51" s="11"/>
-      <c r="D51" s="11"/>
-      <c r="E51" s="11"/>
-      <c r="F51" s="11"/>
-      <c r="G51" s="11"/>
-      <c r="H51" s="11"/>
-      <c r="I51" s="49"/>
-      <c r="J51" s="49"/>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" s="51"/>
     </row>
-    <row r="52" spans="1:10" s="53" customFormat="1" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="B52" s="49"/>
-      <c r="C52" s="49"/>
-      <c r="D52" s="49"/>
-      <c r="E52" s="49"/>
-      <c r="F52" s="49"/>
-      <c r="G52" s="49"/>
-      <c r="H52" s="49"/>
-      <c r="I52" s="49"/>
-      <c r="J52" s="49"/>
-    </row>
-    <row r="53" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="2" t="s">
-        <v>41</v>
-      </c>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" s="51"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A62:A63"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
-  <pageSetup scale="69" orientation="portrait" useFirstPageNumber="1" r:id="rId1"/>
+  <pageSetup scale="62" orientation="portrait" useFirstPageNumber="1" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C- &amp;P -</oddHeader>
   </headerFooter>

</xml_diff>